<commit_message>
auto: snapshot 2026-07-25 05:30:29
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -463,11 +463,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-25 13:00:13</t>
+          <t>Timestamp: 2026-07-25 13:30:29</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0</v>
+        <v>720</v>
       </c>
     </row>
     <row r="3">
@@ -884,7 +884,7 @@
         </is>
       </c>
       <c r="B30" s="3" t="n">
-        <v>14213</v>
+        <v>14333</v>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
@@ -899,7 +899,7 @@
         </is>
       </c>
       <c r="B31" s="3" t="n">
-        <v>18229</v>
+        <v>18349</v>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
@@ -944,7 +944,7 @@
         </is>
       </c>
       <c r="B34" s="3" t="n">
-        <v>17344</v>
+        <v>17584</v>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
@@ -1139,7 +1139,7 @@
         </is>
       </c>
       <c r="B47" s="3" t="n">
-        <v>9506</v>
+        <v>9626</v>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
@@ -1259,7 +1259,7 @@
         </is>
       </c>
       <c r="B55" s="3" t="n">
-        <v>8695</v>
+        <v>8815</v>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-26 05:00:11
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="2026-07-25" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="2026-07-26" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1319,4 +1320,892 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105) | S62</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-07-26 13:00:10</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>33995</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>I Am Dead  @_@</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>NAOR</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>840</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>70</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>+60</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>DangerousEX</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Xylota X Neverlose</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>4257</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>+20</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>MATHEMATRICK</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Tuyu|Fortuners</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>7912</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Khakashi Hatake</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Kosaki</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Prince G™</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>5944</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>ASHBORN™</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Nabila|Fortuners</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>7282</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>4844</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>+1544</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Ryujin Senju™</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>3609</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>19202</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>+4869</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>ZenithEX</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>23365</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+5016</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Meru™</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>22877</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>+5293</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Signature</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Sesshomaru</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>1455</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>2623</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>57</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Flarekaze |Fortuners</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>8124</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>2646</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>+1200</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Breaker LITE</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>15003</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>+5377</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Snoopy | Kokyotosu</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>1080</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Arya</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Morrissey</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>14502</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>+2752</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>20884</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+4724</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>1430</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>1590</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Rood</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>191</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>11095</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+2280</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>+20</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>951</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
auto: snapshot 2026-07-26 05:30:31
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -1352,11 +1352,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-26 13:00:10</t>
+          <t>Timestamp: 2026-07-26 13:30:30</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>33995</v>
+        <v>1285</v>
       </c>
     </row>
     <row r="3">
@@ -1773,11 +1773,11 @@
         </is>
       </c>
       <c r="B30" s="3" t="n">
-        <v>19202</v>
+        <v>19442</v>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>+4869</t>
+          <t>+5109</t>
         </is>
       </c>
     </row>
@@ -1788,11 +1788,11 @@
         </is>
       </c>
       <c r="B31" s="3" t="n">
-        <v>23365</v>
+        <v>23725</v>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>+5016</t>
+          <t>+5376</t>
         </is>
       </c>
     </row>
@@ -1833,11 +1833,11 @@
         </is>
       </c>
       <c r="B34" s="3" t="n">
-        <v>22877</v>
+        <v>23237</v>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>+5293</t>
+          <t>+5653</t>
         </is>
       </c>
     </row>
@@ -2028,11 +2028,11 @@
         </is>
       </c>
       <c r="B47" s="3" t="n">
-        <v>15003</v>
+        <v>15243</v>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>+5377</t>
+          <t>+5617</t>
         </is>
       </c>
     </row>
@@ -2148,11 +2148,11 @@
         </is>
       </c>
       <c r="B55" s="3" t="n">
-        <v>11095</v>
+        <v>11180</v>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>+2280</t>
+          <t>+2365</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-27 05:00:13
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="2026-07-25" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="2026-07-26" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="2026-07-27" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2208,4 +2209,892 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105) | S62</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-07-27 13:00:13</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>I Am Dead  @_@</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>NAOR</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>840</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>118</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>+48</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>DangerousEX</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Xylota X Neverlose</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>4539</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>+282</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>MATHEMATRICK</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Tuyu|Fortuners</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>7912</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Khakashi Hatake</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Kosaki</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Prince G™</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>5944</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>ASHBORN™</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Nabila|Fortuners</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>7282</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>5684</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>+840</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Ryujin Senju™</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>3609</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>23570</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>+4128</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>ZenithEX</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>31157</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+7432</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Meru™</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>28221</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>+4984</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Signature</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Sesshomaru</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>1455</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>2651</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>+28</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>57</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Flarekaze |Fortuners</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>8124</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>2646</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Breaker LITE</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>15243</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Snoopy | Kokyotosu</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>1080</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Arya</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Morrissey</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>17646</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>+3144</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>26967</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+6083</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>1430</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>1590</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Rood</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>1631</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>+1440</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>13429</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+2249</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>951</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
auto: snapshot 2026-07-27 05:31:15
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -2241,11 +2241,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-27 13:00:13</t>
+          <t>Timestamp: 2026-07-27 13:31:14</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0</v>
+        <v>252</v>
       </c>
     </row>
     <row r="3">
@@ -2962,11 +2962,11 @@
         </is>
       </c>
       <c r="B50" s="3" t="n">
-        <v>17646</v>
+        <v>17814</v>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>+3144</t>
+          <t>+3312</t>
         </is>
       </c>
     </row>
@@ -2977,11 +2977,11 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>26967</v>
+        <v>27051</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+6083</t>
+          <t>+6167</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-28 05:00:10
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -10,6 +10,7 @@
     <sheet name="2026-07-25" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="2026-07-26" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="2026-07-27" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="2026-07-28" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3097,4 +3098,892 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105) | S62</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-07-28 13:00:09</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>I Am Dead  @_@</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>NAOR</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>840</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>132</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>+14</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>+6</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>DangerousEX</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Xylota X Neverlose</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>5379</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>+840</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>MATHEMATRICK</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Tuyu|Fortuners</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>7912</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Khakashi Hatake</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Kosaki</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Prince G™</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>7624</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>+1680</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>ASHBORN™</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Nabila|Fortuners</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>7282</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>5684</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Ryujin Senju™</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>3609</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>24578</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>+1008</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>ZenithEX</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>35318</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+4161</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Meru™</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>29733</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>+1512</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Signature</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Yamato Senju</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>1455</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>2651</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>57</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Flarekaze |Fortuners</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>8124</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>3066</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>+420</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Breaker LITE</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>15243</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Snoopy | Kokyotosu</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>1080</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Arya</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Morrissey</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>19481</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>+1667</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>30856</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+3805</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>1430</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>1590</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Rood</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>1631</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>14185</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+756</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>3333</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>+3313</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>951</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
auto: snapshot 2026-07-28 05:29:21
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -3130,11 +3130,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-28 13:00:09</t>
+          <t>Timestamp: 2026-07-28 13:29:20</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0</v>
+        <v>336</v>
       </c>
     </row>
     <row r="3">
@@ -3551,11 +3551,11 @@
         </is>
       </c>
       <c r="B30" s="3" t="n">
-        <v>24578</v>
+        <v>24662</v>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>+1008</t>
+          <t>+1092</t>
         </is>
       </c>
     </row>
@@ -3566,11 +3566,11 @@
         </is>
       </c>
       <c r="B31" s="3" t="n">
-        <v>35318</v>
+        <v>35402</v>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>+4161</t>
+          <t>+4245</t>
         </is>
       </c>
     </row>
@@ -3866,11 +3866,11 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>30856</v>
+        <v>30940</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+3805</t>
+          <t>+3889</t>
         </is>
       </c>
     </row>
@@ -3956,11 +3956,11 @@
         </is>
       </c>
       <c r="B57" s="3" t="n">
-        <v>3333</v>
+        <v>3417</v>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>+3313</t>
+          <t>+3397</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-28 05:59:38
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -3130,11 +3130,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-28 13:30:28</t>
+          <t>Timestamp: 2026-07-28 13:59:37</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>336</v>
+        <v>756</v>
       </c>
     </row>
     <row r="3">
@@ -3566,11 +3566,11 @@
         </is>
       </c>
       <c r="B31" s="3" t="n">
-        <v>35402</v>
+        <v>35486</v>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>+4245</t>
+          <t>+4329</t>
         </is>
       </c>
     </row>
@@ -3611,11 +3611,11 @@
         </is>
       </c>
       <c r="B34" s="3" t="n">
-        <v>29733</v>
+        <v>29901</v>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>+1512</t>
+          <t>+1680</t>
         </is>
       </c>
     </row>
@@ -3866,11 +3866,11 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>30940</v>
+        <v>31024</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+3889</t>
+          <t>+3973</t>
         </is>
       </c>
     </row>
@@ -3956,11 +3956,11 @@
         </is>
       </c>
       <c r="B57" s="3" t="n">
-        <v>3417</v>
+        <v>3501</v>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>+3397</t>
+          <t>+3481</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-29 05:00:11
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -11,6 +11,7 @@
     <sheet name="2026-07-26" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="2026-07-27" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="2026-07-28" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="2026-07-29" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3986,4 +3987,892 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105) | S62</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-07-29 13:00:10</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>I Am Dead  @_@</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>NAOR</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>840</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>142</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>+10</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>DangerousEX</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Xylota X Neverlose</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>5379</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>MATHEMATRICK</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Tuyu|Fortuners</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>7912</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Khakashi Hatake</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Kosaki</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Prince G™</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>8848</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>+1224</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>ASHBORN™</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Nabila|Fortuners</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>7282</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>6068</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>+384</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Ryujin Senju™</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>4449</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>+840</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>26978</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>+2316</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>ZenithEX</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>38891</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+3405</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Meru™</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>32643</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>+2742</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Signature</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Yamato Senju</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>1455</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>2651</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>57</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Flarekaze |Fortuners</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>8124</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>3066</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Breaker LITE</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>15243</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Snoopy | Kokyotosu</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>1080</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Arya</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Morrissey</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>20727</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>+1246</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>34490</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+3466</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>1430</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>1890</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Rood</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>1631</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>14857</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+672</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>6671</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>+3170</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>951</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
auto: snapshot 2026-07-29 05:30:25
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -4019,11 +4019,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-29 13:00:10</t>
+          <t>Timestamp: 2026-07-29 13:30:24</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0</v>
+        <v>480</v>
       </c>
     </row>
     <row r="3">
@@ -4305,11 +4305,11 @@
         </is>
       </c>
       <c r="B21" s="3" t="n">
-        <v>8848</v>
+        <v>8968</v>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>+1224</t>
+          <t>+1344</t>
         </is>
       </c>
     </row>
@@ -4500,11 +4500,11 @@
         </is>
       </c>
       <c r="B34" s="3" t="n">
-        <v>32643</v>
+        <v>32763</v>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>+2742</t>
+          <t>+2862</t>
         </is>
       </c>
     </row>
@@ -4755,11 +4755,11 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>34490</v>
+        <v>34550</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+3466</t>
+          <t>+3526</t>
         </is>
       </c>
     </row>
@@ -4845,11 +4845,11 @@
         </is>
       </c>
       <c r="B57" s="3" t="n">
-        <v>6671</v>
+        <v>6851</v>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>+3170</t>
+          <t>+3350</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-29 05:36:17
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -4019,11 +4019,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-29 13:30:24</t>
+          <t>Timestamp: 2026-07-29 13:36:16</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>480</v>
+        <v>600</v>
       </c>
     </row>
     <row r="3">
@@ -4755,11 +4755,11 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>34550</v>
+        <v>34610</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+3526</t>
+          <t>+3586</t>
         </is>
       </c>
     </row>
@@ -4845,11 +4845,11 @@
         </is>
       </c>
       <c r="B57" s="3" t="n">
-        <v>6851</v>
+        <v>6911</v>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>+3350</t>
+          <t>+3410</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-30 05:00:12
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -12,6 +12,7 @@
     <sheet name="2026-07-27" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="2026-07-28" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="2026-07-29" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="2026-07-30" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4875,4 +4876,892 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105) | S62</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-07-30 13:00:12</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>16876</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>I Am Dead  @_@</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>NAOR</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>840</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>152</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>+10</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>DangerousEX</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Xylota X Neverlose</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>5379</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>MATHEMATRICK</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Tuyu|Fortuners</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>7912</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Khakashi Hatake</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Kosaki</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Prince G™</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>10390</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>+1422</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>ASHBORN™</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Nabila|Fortuners</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>7282</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>6368</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Ryujin Senju™</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>4749</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>29078</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>+2100</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>ZenithEX</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>41486</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+2595</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Meru™</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>35343</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>+2580</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Signature</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Sesshomaru</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>1545</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>2651</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>57</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Flarekaze |Fortuners</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>8124</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>3366</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Breaker LITE</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>15243</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Snoopy | Kokyotosu</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>2040</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>+960</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Arya</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Morrissey</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>21027</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>37370</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+2760</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>1430</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>1890</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Rood</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>1631</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>15217</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+360</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>9110</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>+2199</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>951</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
auto: snapshot 2026-07-30 05:30:30
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -4908,11 +4908,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-30 13:00:12</t>
+          <t>Timestamp: 2026-07-30 13:30:30</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>16876</v>
+        <v>17056</v>
       </c>
     </row>
     <row r="3">
@@ -5344,11 +5344,11 @@
         </is>
       </c>
       <c r="B31" s="3" t="n">
-        <v>41486</v>
+        <v>41546</v>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>+2595</t>
+          <t>+2655</t>
         </is>
       </c>
     </row>
@@ -5644,11 +5644,11 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>37370</v>
+        <v>37430</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+2760</t>
+          <t>+2820</t>
         </is>
       </c>
     </row>
@@ -5734,11 +5734,11 @@
         </is>
       </c>
       <c r="B57" s="3" t="n">
-        <v>9110</v>
+        <v>9170</v>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>+2199</t>
+          <t>+2259</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-31 05:00:10
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -13,6 +13,7 @@
     <sheet name="2026-07-28" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="2026-07-29" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="2026-07-30" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="2026-07-31" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -5764,4 +5765,892 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105) | S62</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-07-31 13:00:10</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>I Am Dead  @_@</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>NAOR</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>840</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>162</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>+10</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>DangerousEX</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Xylota X Neverlose</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>5670</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>+291</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>320</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>MATHEMATRICK</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>250</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>+250</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Tuyu|Fortuners</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>7912</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Khakashi Hatake</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Kosaki</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Prince G™</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>11660</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>+1270</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>ASHBORN™</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Nabila|Fortuners</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>7282</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>6668</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Ryujin Senju™</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>5049</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>30908</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>+1830</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>ZenithEX</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>44294</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+2748</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Meru™</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>37122</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>+1779</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Signature</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Sesshomaru</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>1545</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>2651</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>57</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Flarekaze |Fortuners</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>8124</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>3366</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Breaker LITE</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>15243</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Snoopy | Kokyotosu</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>2400</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>+360</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Arya</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Morrissey</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>21037</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>+10</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>40070</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+2640</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>1430</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>1890</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Rood</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>1631</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>15733</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+516</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>300</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>11669</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>+2499</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>1262</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>+311</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
auto: snapshot 2026-07-31 05:30:31
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -5797,11 +5797,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-31 13:00:10</t>
+          <t>Timestamp: 2026-07-31 13:30:30</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0</v>
+        <v>300</v>
       </c>
     </row>
     <row r="3">
@@ -6218,11 +6218,11 @@
         </is>
       </c>
       <c r="B30" s="3" t="n">
-        <v>30908</v>
+        <v>30968</v>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>+1830</t>
+          <t>+1890</t>
         </is>
       </c>
     </row>
@@ -6233,11 +6233,11 @@
         </is>
       </c>
       <c r="B31" s="3" t="n">
-        <v>44294</v>
+        <v>44354</v>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>+2748</t>
+          <t>+2808</t>
         </is>
       </c>
     </row>
@@ -6278,11 +6278,11 @@
         </is>
       </c>
       <c r="B34" s="3" t="n">
-        <v>37122</v>
+        <v>37182</v>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>+1779</t>
+          <t>+1839</t>
         </is>
       </c>
     </row>
@@ -6533,11 +6533,11 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>40070</v>
+        <v>40130</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+2640</t>
+          <t>+2700</t>
         </is>
       </c>
     </row>
@@ -6623,11 +6623,11 @@
         </is>
       </c>
       <c r="B57" s="3" t="n">
-        <v>11669</v>
+        <v>11729</v>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>+2499</t>
+          <t>+2559</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-01 05:00:12
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -14,6 +14,7 @@
     <sheet name="2026-07-29" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="2026-07-30" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="2026-07-31" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="2026-08-01" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -6653,4 +6654,892 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105) | S62</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-01 13:00:12</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>12526</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>I Am Dead  @_@</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>NAOR</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>840</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>162</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>DangerousEX</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Xylota X Neverlose</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>5970</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>320</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>MATHEMATRICK</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>250</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Tuyu|Fortuners</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>7912</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Khakashi Hatake</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Kosaki</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Prince G™</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>11960</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>ASHBORN™</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Nabila|Fortuners</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>7282</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>6968</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Ryujin Senju™</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>5049</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>32948</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>+1980</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>ZenithEX</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>45854</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+1500</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Meru™</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>39162</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>+1980</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Signature</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Sesshomaru</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>1545</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>2651</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>57</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Flarekaze |Fortuners</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>8124</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>3666</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Breaker LITE</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>15243</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Snoopy | Kokyotosu</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>2400</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Arya</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Morrissey</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>21799</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>+762</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>41993</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+1863</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>1430</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>1890</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Rood</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>1631</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>16784</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+1051</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>300</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>13619</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>+1890</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>1262</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
auto: snapshot 2026-08-01 05:30:27
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -6686,11 +6686,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-01 13:00:12</t>
+          <t>Timestamp: 2026-08-01 13:30:26</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>12526</v>
+        <v>420</v>
       </c>
     </row>
     <row r="3">
@@ -7452,11 +7452,11 @@
         </is>
       </c>
       <c r="B53" s="3" t="n">
-        <v>1890</v>
+        <v>1910</v>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+20</t>
         </is>
       </c>
     </row>
@@ -7482,11 +7482,11 @@
         </is>
       </c>
       <c r="B55" s="3" t="n">
-        <v>16784</v>
+        <v>17184</v>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>+1051</t>
+          <t>+1451</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-02 05:00:11
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -15,6 +15,7 @@
     <sheet name="2026-07-30" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="2026-07-31" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="2026-08-01" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="2026-08-02" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -7542,4 +7543,892 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105) | S62</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-02 13:00:10</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>17860</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>I Am Dead  @_@</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>NAOR</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>840</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>282</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>+120</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>DangerousEX</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Xylota x [NvL]</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>6570</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>320</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>MATHEMATRICK</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>250</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Tuyu|Fortuners</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>7912</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Khakashi Hatake</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Kosaki</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>1793</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>+1793</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Prince G™</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>11960</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>ASHBORN™</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Nabila|Fortuners</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>7282</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>7568</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Ryujin Senju™</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>5049</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>32948</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>ZenithEX</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>45874</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+20</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Meru™</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>1376</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>+1376</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>39762</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Signature</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Sesshomaru</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>3584</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>+2039</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>2651</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>57</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Flarekaze |Fortuners</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>8124</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>3666</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Breaker LITE</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>15243</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Snoopy | Kokyotosu</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>2400</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Ary</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Morrissey</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>23163</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>+1364</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>45602</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+3609</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>1430</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>1910</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Rood</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>1631</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>21303</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+4119</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>900</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>13619</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>1862</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
auto: snapshot 2026-08-02 05:30:28
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -7575,11 +7575,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-02 13:00:10</t>
+          <t>Timestamp: 2026-08-02 13:30:27</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>17860</v>
+        <v>245</v>
       </c>
     </row>
     <row r="3">
@@ -8311,11 +8311,11 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>45602</v>
+        <v>45722</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+3609</t>
+          <t>+3729</t>
         </is>
       </c>
     </row>
@@ -8371,11 +8371,11 @@
         </is>
       </c>
       <c r="B55" s="3" t="n">
-        <v>21303</v>
+        <v>21428</v>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>+4119</t>
+          <t>+4244</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-03 05:00:10
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -16,6 +16,7 @@
     <sheet name="2026-07-31" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="2026-08-01" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="2026-08-02" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="2026-08-03" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1329,6 +1330,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105) | S62</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-03 13:00:10</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>22641</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>I Am Dead  @_@</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>NAOR</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>840</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>582</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>DangerousEX</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Xylota x [NvL]</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>7290</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>+720</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>320</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>MATHEMATRICK</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>250</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Tuyu|Fortuners</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>7912</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Khakashi Hatake</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Kosaki</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>5399</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>+3606</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Prince G™</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>11960</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>ASHBORN™</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Nabila|Fortuners</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>7282</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>8168</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Ryujin Senju™</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>5049</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>32948</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>ZenithEX</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>46714</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+840</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Meru™</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>4123</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>+2747</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>39762</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Signature</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Sesshomaru</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>7304</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>+3720</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>2651</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>57</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Flarekaze |Fortuners</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>8124</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>3666</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Breaker LITE</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>15243</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Kokyotosu</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>2400</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Arya</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Morri§ey</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>24344</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>50729</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+5007</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>1430</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>1910</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Rood</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>1631</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>25103</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+3675</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>900</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>13619</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>1862</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-03 05:01:57
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -1360,11 +1360,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-03 13:00:10</t>
+          <t>Timestamp: 2026-08-03 13:01:56</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>22641</v>
+        <v>60</v>
       </c>
     </row>
     <row r="3">
@@ -1886,11 +1886,11 @@
         </is>
       </c>
       <c r="B37" s="3" t="n">
-        <v>7304</v>
+        <v>7364</v>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>+3720</t>
+          <t>+3780</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-03 05:30:26
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -1360,11 +1360,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-03 13:01:56</t>
+          <t>Timestamp: 2026-08-03 13:30:25</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>60</v>
+        <v>120</v>
       </c>
     </row>
     <row r="3">
@@ -1631,11 +1631,11 @@
         </is>
       </c>
       <c r="B20" s="3" t="n">
-        <v>5399</v>
+        <v>5459</v>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>+3606</t>
+          <t>+3666</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-04 05:00:01
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -17,6 +17,7 @@
     <sheet name="2026-08-01" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="2026-08-02" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="2026-08-03" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="2026-08-04" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2218,6 +2219,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105) | S62</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-04 13:00:00</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>10516</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>I Am Dead  @_@</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>NAOR</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>840</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>592</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>+10</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>DangerousEX</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Xylota x [NvL]</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>7650</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>+360</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>320</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>611</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>+611</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>MATHEMATRICK</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>250</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Tuyu|Fortuners</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>7912</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Khakashi Hatake</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Kosaki</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>6479</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>+1020</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Prince G™</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>11960</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>ASHBORN™</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Nabila|Fortuners</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>7282</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>8468</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Ryujin Senju™</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>5589</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>+540</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>32948</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>ZenithEX</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>46714</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Meru™</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>5403</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>+1280</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>39762</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Signature</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Sesshomaru</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>8384</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>+1020</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>2651</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>57</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Flarekaze |Fortuners</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>8124</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>3666</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Breaker LITE</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>15243</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Kokyotosu</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>2400</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Arya</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>300</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Morri§ey</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>24344</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>53004</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+2275</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>1430</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>2040</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>+130</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Rood</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>1631</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>27653</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+2550</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>900</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>13619</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>1862</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-04 05:00:21
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -2249,11 +2249,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-04 13:00:00</t>
+          <t>Timestamp: 2026-08-04 13:00:20</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>10516</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
auto: snapshot 2026-08-04 05:30:08
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -2249,11 +2249,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-04 13:00:20</t>
+          <t>Timestamp: 2026-08-04 13:30:08</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
     </row>
     <row r="3">
@@ -2985,11 +2985,11 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>53004</v>
+        <v>53064</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+2275</t>
+          <t>+2335</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-05 05:00:09
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -18,6 +18,7 @@
     <sheet name="2026-08-02" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="2026-08-03" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="2026-08-04" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="2026-08-05" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3107,6 +3108,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105) | S62</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-05 13:00:09</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>11472</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>I Am Dead  @_@</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>NAOR</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>840</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>592</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>DangerousEX</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Xylota x [NvL]</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>8010</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>+360</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>320</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>621</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>+10</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>MATHEMATRICK</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>250</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Tuyu|Fortuners</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>7912</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Khakashi Hatake</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Kosaki</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>7970</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>+1491</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Prince G™</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>11960</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>ASHBORN™</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>+50</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Nabila|Fortuners</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>7282</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>8768</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Ryujin Senju™</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>5589</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>32948</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>ZenithEX</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>47074</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+360</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Meru™</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>6876</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>+1473</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>39762</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Signature</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Sesshomaru</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>9897</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>+1513</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>2651</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>57</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Flarekaze |Fortuners</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>8124</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>3666</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Breaker LITE</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>15243</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Kokyotosu</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>2400</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Arya</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>300</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Morri§ey</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>24344</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>55884</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+2820</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>1430</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>2060</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>+20</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Rood</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>1631</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>29468</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+1815</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>900</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>14819</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>+1200</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>1862</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-05 05:29:08
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -3138,11 +3138,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-05 13:00:09</t>
+          <t>Timestamp: 2026-08-05 13:29:07</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>11472</v>
+        <v>320</v>
       </c>
     </row>
     <row r="3">
@@ -3874,11 +3874,11 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>55884</v>
+        <v>55944</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+2820</t>
+          <t>+2880</t>
         </is>
       </c>
     </row>
@@ -3964,11 +3964,11 @@
         </is>
       </c>
       <c r="B57" s="3" t="n">
-        <v>14819</v>
+        <v>15079</v>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>+1200</t>
+          <t>+1460</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-05 05:59:21
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -3138,11 +3138,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-05 13:30:20</t>
+          <t>Timestamp: 2026-08-05 13:59:21</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>320</v>
+        <v>497</v>
       </c>
     </row>
     <row r="3">
@@ -3874,11 +3874,11 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>55944</v>
+        <v>56004</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+2880</t>
+          <t>+2940</t>
         </is>
       </c>
     </row>
@@ -3934,11 +3934,11 @@
         </is>
       </c>
       <c r="B55" s="3" t="n">
-        <v>29468</v>
+        <v>29525</v>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>+1815</t>
+          <t>+1872</t>
         </is>
       </c>
     </row>
@@ -3964,11 +3964,11 @@
         </is>
       </c>
       <c r="B57" s="3" t="n">
-        <v>15079</v>
+        <v>15139</v>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>+1460</t>
+          <t>+1520</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-06 05:00:12
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -19,6 +19,7 @@
     <sheet name="2026-08-03" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="2026-08-04" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="2026-08-05" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="2026-08-06" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3996,6 +3997,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105) | S62</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-06 13:00:12</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>17096</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>300K Tokens LetsGo!</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>NAOR</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>840</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>592</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>DangerousEX</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Xylota x [NvL]</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>8310</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>320</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>621</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>MATHEMATRICK</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>250</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Tuyu|Fortuners</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>7912</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Khakashi Hatake</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>+12</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Kosaki</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>9422</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>+1452</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Prince G™</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>11960</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>ASHBORN™</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Nabila|Fortuners</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>7282</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>9068</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Ryujin Senju™</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>5589</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>32948</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>ZenithEX</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>47746</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+672</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Meru™</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>8613</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>+1737</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>39762</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Signature</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>350K All in</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>11534</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>2651</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>57</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Flarekaze |Fortuners</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>8124</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>3666</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Breaker LITE</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>16851</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>+1608</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Kokyotosu</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>2400</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Ary</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>300</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Morri§ey</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>24354</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>+10</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>59004</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+3000</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>1430</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>2060</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Rood</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>1631</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>32444</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+2919</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>900</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>18091</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>+2952</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>1862</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-06 05:30:25
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -4027,11 +4027,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-06 13:00:12</t>
+          <t>Timestamp: 2026-08-06 13:30:25</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>17096</v>
+        <v>290</v>
       </c>
     </row>
     <row r="3">
@@ -4463,11 +4463,11 @@
         </is>
       </c>
       <c r="B31" s="3" t="n">
-        <v>47746</v>
+        <v>47806</v>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>+672</t>
+          <t>+732</t>
         </is>
       </c>
     </row>
@@ -4703,11 +4703,11 @@
         </is>
       </c>
       <c r="B47" s="3" t="n">
-        <v>16851</v>
+        <v>16911</v>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>+1608</t>
+          <t>+1668</t>
         </is>
       </c>
     </row>
@@ -4763,11 +4763,11 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>59004</v>
+        <v>59054</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+3000</t>
+          <t>+3050</t>
         </is>
       </c>
     </row>
@@ -4823,11 +4823,11 @@
         </is>
       </c>
       <c r="B55" s="3" t="n">
-        <v>32444</v>
+        <v>32504</v>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>+2919</t>
+          <t>+2979</t>
         </is>
       </c>
     </row>
@@ -4853,11 +4853,11 @@
         </is>
       </c>
       <c r="B57" s="3" t="n">
-        <v>18091</v>
+        <v>18151</v>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>+2952</t>
+          <t>+3012</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-06 05:46:16
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -4027,11 +4027,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-06 13:30:25</t>
+          <t>Timestamp: 2026-08-06 13:46:15</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>290</v>
+        <v>420</v>
       </c>
     </row>
     <row r="3">
@@ -4703,11 +4703,11 @@
         </is>
       </c>
       <c r="B47" s="3" t="n">
-        <v>16911</v>
+        <v>16971</v>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>+1668</t>
+          <t>+1728</t>
         </is>
       </c>
     </row>
@@ -4763,11 +4763,11 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>59054</v>
+        <v>59124</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+3050</t>
+          <t>+3120</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-07 05:00:11
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -20,6 +20,7 @@
     <sheet name="2026-08-04" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="2026-08-05" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="2026-08-06" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="2026-08-07" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4885,6 +4886,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105) | S62</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-07 13:00:10</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>15147</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>300K Tokens LetsGo!</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>NAOR</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>840</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>592</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>DangerousEX</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Xylota x [NvL]</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>8310</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>320</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>621</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>MATHEMATRICK</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>250</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Tuyu|Fortuners</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>7912</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Khakashi Hatake</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>+2</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Kosaki</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>9422</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Prince G™</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>11960</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>ASHBORN™</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Nabila|Fortuners</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>7282</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>9908</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>+840</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Ryujin Senju™</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>5589</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>32948</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>ZenithEX</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>48366</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+560</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Meru™</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>8613</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>39762</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Signature</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>350K All in</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>11534</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>2651</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>57</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Flarekaze |Fortuners</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>8124</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Raiden</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>3666</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Breaker LITE</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>20222</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>+3251</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Kokyotosu</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>2400</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Ary</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>300</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Morri§ey</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>24354</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>62816</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+3692</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>1430</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>2060</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Rood</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>1631</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>35201</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+2697</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>900</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>21836</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>+3685</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>1862</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-07 05:30:27
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -4916,11 +4916,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-07 13:00:10</t>
+          <t>Timestamp: 2026-08-07 13:30:26</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>15147</v>
+        <v>250</v>
       </c>
     </row>
     <row r="3">
@@ -5592,11 +5592,11 @@
         </is>
       </c>
       <c r="B47" s="3" t="n">
-        <v>20222</v>
+        <v>20282</v>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>+3251</t>
+          <t>+3311</t>
         </is>
       </c>
     </row>
@@ -5652,11 +5652,11 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>62816</v>
+        <v>62876</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+3692</t>
+          <t>+3752</t>
         </is>
       </c>
     </row>
@@ -5682,11 +5682,11 @@
         </is>
       </c>
       <c r="B53" s="3" t="n">
-        <v>2060</v>
+        <v>2070</v>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+10</t>
         </is>
       </c>
     </row>
@@ -5712,11 +5712,11 @@
         </is>
       </c>
       <c r="B55" s="3" t="n">
-        <v>35201</v>
+        <v>35261</v>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>+2697</t>
+          <t>+2757</t>
         </is>
       </c>
     </row>
@@ -5742,11 +5742,11 @@
         </is>
       </c>
       <c r="B57" s="3" t="n">
-        <v>21836</v>
+        <v>21896</v>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>+3685</t>
+          <t>+3745</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-08 05:00:11
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -21,6 +21,7 @@
     <sheet name="2026-08-05" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="2026-08-06" sheetId="13" state="visible" r:id="rId13"/>
     <sheet name="2026-08-07" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="2026-08-08" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -5774,6 +5775,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105) | S62</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-08 13:00:11</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>18324</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>961</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>+961</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>300K Tokens LetsGo!</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>NAOR</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>840</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>1389</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>+797</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>DangerousEX</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Xylota x [NvL]</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>9326</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>+1016</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>320</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>621</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>MATHEMATRICK</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>251</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>+1</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Tuyu|Fortuners</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>7912</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Khakashi Hatake</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>34</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>+20</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Kosaki</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>9422</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Prince G™</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>11960</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>420</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>+420</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>ASHBORN™</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Nabila|Fortuners</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>7282</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>10581</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>+673</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Ryujin Senju™</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>5589</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>32948</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>BlacKoreana O</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>48823</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Meru™</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>8613</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>39762</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Signature</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>350K All in</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>11534</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>2651</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>778</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>+778</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>57</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Flarekaze |Fortuners</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>8124</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Raiden</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>3666</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Breaker LITE</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>23025</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>+2743</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Kokyotosu</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>2400</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Ary</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>766</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>+466</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Morri§ey</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>25962</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>+1608</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>65906</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+3030</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>1430</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>2070</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Rood</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>1631</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>37509</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+2248</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>900</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>24752</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>+2856</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>1862</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-08 05:30:24
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -5805,11 +5805,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-08 13:00:11</t>
+          <t>Timestamp: 2026-08-08 13:30:23</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>18324</v>
+        <v>240</v>
       </c>
     </row>
     <row r="3">
@@ -6481,11 +6481,11 @@
         </is>
       </c>
       <c r="B47" s="3" t="n">
-        <v>23025</v>
+        <v>23145</v>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>+2743</t>
+          <t>+2863</t>
         </is>
       </c>
     </row>
@@ -6541,11 +6541,11 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>65906</v>
+        <v>66026</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+3030</t>
+          <t>+3150</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-08 05:39:53
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -5805,11 +5805,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-08 13:30:23</t>
+          <t>Timestamp: 2026-08-08 13:39:52</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>240</v>
+        <v>581</v>
       </c>
     </row>
     <row r="3">
@@ -6481,11 +6481,11 @@
         </is>
       </c>
       <c r="B47" s="3" t="n">
-        <v>23145</v>
+        <v>23265</v>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>+2863</t>
+          <t>+2983</t>
         </is>
       </c>
     </row>
@@ -6601,11 +6601,11 @@
         </is>
       </c>
       <c r="B55" s="3" t="n">
-        <v>37509</v>
+        <v>37730</v>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>+2248</t>
+          <t>+2469</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-09 05:00:12
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -22,6 +22,7 @@
     <sheet name="2026-08-06" sheetId="13" state="visible" r:id="rId13"/>
     <sheet name="2026-08-07" sheetId="14" state="visible" r:id="rId14"/>
     <sheet name="2026-08-08" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="2026-08-09" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -6663,6 +6664,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105) | S62</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-09 13:00:12</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>29770</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>+28809</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>300K Tokens LetsGo!</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>25009</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>+24989</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>NAOR</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>26049</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>+25209</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>21021</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>+19632</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>23879</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>+23873</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>29023</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>+29023</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>£_Darkz_£</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>19050</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>DangerousEX</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>16131</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>+16131</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Xylota x [NvL]</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>39805</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>+30479</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>15428</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>+15108</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>18006</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>+17385</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>MATHEMATRICK</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>29311</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>+29311</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>21573</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>+21322</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>25802</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>+25802</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Khakashi Hatake</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>28796</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>+28796</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>28908</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>+28874</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Kosaki</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>37257</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>+27835</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Prince G™</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>36707</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>+24747</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>14558</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>+14558</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>27667</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>+27667</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>27423</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>+27003</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>ASHBORN™</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>28409</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>+28359</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Nabila|Fortuners</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>35328</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>+28046</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>39401</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>+28820</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Ryujin Senju™</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>27598</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>+22009</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>28725</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>+28725</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>59848</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>+26900</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>BlacKoreana O</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>74851</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+26028</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>29535</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>+29535</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Meru™</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>23520</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>+14907</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>56954</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>+17192</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Signature</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>23635</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>+23635</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>23619</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>+23619</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Sesshomaru</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>33785</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>22402</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>+19751</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>29661</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>+28883</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>28816</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>+28759</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Flarekaze |Fortuners</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>23421</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>+15297</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Raiden</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>26957</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>+26957</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>30793</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>+27127</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>27113</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>+27113</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>28524</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>+28524</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>28683</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>+28647</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Breaker LITE</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>55017</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>+31752</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Kokyotosu</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>30999</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>+28599</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Ary</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>29493</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>+28727</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Morri§ey</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>47422</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>+21460</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>96586</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+30560</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>29715</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>+28285</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>30822</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>+28752</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Rood</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>23204</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>+21573</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>56793</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+19063</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>19547</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>+18647</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>54191</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>+29439</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>27604</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>+25742</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-10 05:00:11
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -23,6 +23,7 @@
     <sheet name="2026-08-07" sheetId="14" state="visible" r:id="rId14"/>
     <sheet name="2026-08-08" sheetId="15" state="visible" r:id="rId15"/>
     <sheet name="2026-08-09" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="2026-08-10" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -7552,6 +7553,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105) | S63</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-10 13:00:10</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>6622</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>NAOR</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>330</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>£_Darkz_£</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>DangerousEX</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Xylota x [NvL]</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>342</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>MATHEMATRICK</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Khakashi Hatake</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Kosaki</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Prince G™</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>786</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>ASHBORN™</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Nabila|Fortuners</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Ryujin Senju™</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>BlacKoreana O</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Meru™</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>683</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Signature</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Sesshomaru</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Flarekaze |Fortuners</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Raiden</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Breaker LITE</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Kokyotosu</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Ary</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Morri§ey</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>783</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>626</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Rood</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>1257</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>1205</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>600</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-10 05:30:25
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -7583,11 +7583,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-10 13:00:10</t>
+          <t>Timestamp: 2026-08-10 13:30:24</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>6622</v>
+        <v>1350</v>
       </c>
     </row>
     <row r="3">
@@ -7734,7 +7734,7 @@
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>342</v>
+        <v>1092</v>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
@@ -7914,7 +7914,7 @@
         </is>
       </c>
       <c r="B24" s="3" t="n">
-        <v>786</v>
+        <v>936</v>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
@@ -8319,7 +8319,7 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>626</v>
+        <v>926</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
@@ -8409,7 +8409,7 @@
         </is>
       </c>
       <c r="B57" s="3" t="n">
-        <v>1205</v>
+        <v>1355</v>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-10 05:54:35
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -7583,11 +7583,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-10 13:30:24</t>
+          <t>Timestamp: 2026-08-10 13:54:34</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>1350</v>
+        <v>1935</v>
       </c>
     </row>
     <row r="3">
@@ -7764,7 +7764,7 @@
         </is>
       </c>
       <c r="B14" s="3" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
@@ -7914,7 +7914,7 @@
         </is>
       </c>
       <c r="B24" s="3" t="n">
-        <v>936</v>
+        <v>990</v>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
@@ -8319,7 +8319,7 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>926</v>
+        <v>932</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
@@ -8379,7 +8379,7 @@
         </is>
       </c>
       <c r="B55" s="3" t="n">
-        <v>1257</v>
+        <v>1557</v>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
@@ -8409,7 +8409,7 @@
         </is>
       </c>
       <c r="B57" s="3" t="n">
-        <v>1355</v>
+        <v>1505</v>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-11 05:00:12
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -24,6 +24,7 @@
     <sheet name="2026-08-08" sheetId="15" state="visible" r:id="rId15"/>
     <sheet name="2026-08-09" sheetId="16" state="visible" r:id="rId16"/>
     <sheet name="2026-08-10" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="2026-08-11" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -8441,6 +8442,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105) | S63</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-11 13:00:11</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>19623</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>NAOR</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>1393</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>+1063</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>£_Darkz_£</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>DangerousEX</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Xylota x [NvL]</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>3146</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>+2054</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>150</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>+75</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>MATHEMATRICK</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Khakashi Hatake</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Kosaki</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Prince G™</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>3055</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>+2065</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>ASHBORN™</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Nabila|Fortuners</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Ryujin Senju™</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>BlacKoreana O</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Meru™</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>683</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Signature</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Sesshomaru</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Flarekaze |Fortuners</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Raiden</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Breaker LITE</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>1080</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>+1080</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Kokyotosu</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Ary</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Morri§ey</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>2306</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>+1523</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>5335</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+4403</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>+19</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Rood</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>2951</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+1394</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>5517</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>+4012</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>600</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-11 05:30:24
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -8472,11 +8472,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-11 13:00:11</t>
+          <t>Timestamp: 2026-08-11 13:30:23</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>19623</v>
+        <v>267</v>
       </c>
     </row>
     <row r="3">
@@ -9193,11 +9193,11 @@
         </is>
       </c>
       <c r="B50" s="3" t="n">
-        <v>2306</v>
+        <v>2391</v>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>+1523</t>
+          <t>+1608</t>
         </is>
       </c>
     </row>
@@ -9208,11 +9208,11 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>5335</v>
+        <v>5419</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+4403</t>
+          <t>+4487</t>
         </is>
       </c>
     </row>
@@ -9313,11 +9313,11 @@
         </is>
       </c>
       <c r="B58" s="3" t="n">
-        <v>600</v>
+        <v>698</v>
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+98</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-12 05:00:11
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -25,6 +25,7 @@
     <sheet name="2026-08-09" sheetId="16" state="visible" r:id="rId16"/>
     <sheet name="2026-08-10" sheetId="17" state="visible" r:id="rId17"/>
     <sheet name="2026-08-11" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="2026-08-12" sheetId="19" state="visible" r:id="rId19"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -9330,6 +9331,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105) | S63</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-12 13:00:10</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>18216</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>NAOR</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>1393</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>1508</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>+1508</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>£_Darkz_£</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>DangerousEX</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Xylota x [NvL]</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>4126</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>+980</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>258</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>+108</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>MATHEMATRICK</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Khakashi Hatake</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Kosaki</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Prince G™</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>6955</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>+3900</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>ASHBORN™</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Nabila|Fortuners</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Ryujin Senju™</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>BlacKoreana O</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Meru™</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>683</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Signature</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Sesshomaru</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Flarekaze |Fortuners</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Raiden</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Breaker LITE</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>4899</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>+3819</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Kokyotosu</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Ary</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Morri§ey</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>4474</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>+2083</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>10430</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+5011</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Rood</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>2951</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>5517</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>1238</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>+540</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-12 05:30:26
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -9361,11 +9361,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-12 13:00:10</t>
+          <t>Timestamp: 2026-08-12 13:30:26</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>18216</v>
+        <v>216</v>
       </c>
     </row>
     <row r="3">
@@ -10037,11 +10037,11 @@
         </is>
       </c>
       <c r="B47" s="3" t="n">
-        <v>4899</v>
+        <v>5007</v>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>+3819</t>
+          <t>+3927</t>
         </is>
       </c>
     </row>
@@ -10097,11 +10097,11 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>10430</v>
+        <v>10538</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+5011</t>
+          <t>+5119</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-12 05:54:01
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -9361,11 +9361,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-12 13:30:26</t>
+          <t>Timestamp: 2026-08-12 13:54:00</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>216</v>
+        <v>432</v>
       </c>
     </row>
     <row r="3">
@@ -10037,11 +10037,11 @@
         </is>
       </c>
       <c r="B47" s="3" t="n">
-        <v>5007</v>
+        <v>5115</v>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>+3927</t>
+          <t>+4035</t>
         </is>
       </c>
     </row>
@@ -10097,11 +10097,11 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>10538</v>
+        <v>10646</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+5119</t>
+          <t>+5227</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-13 05:00:14
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -26,6 +26,7 @@
     <sheet name="2026-08-10" sheetId="17" state="visible" r:id="rId17"/>
     <sheet name="2026-08-11" sheetId="18" state="visible" r:id="rId18"/>
     <sheet name="2026-08-12" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="2026-08-13" sheetId="20" state="visible" r:id="rId20"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -11107,6 +11108,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105) | S63</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-13 13:00:13</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>14900</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>NAOR</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>1956</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>+563</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>+36</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>3452</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>+1944</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>£_Darkz_£</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>DangerousEX</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Xylota x [NvL]</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>6394</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>+2268</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>258</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>MATHEMATRICK</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Khakashi Hatake</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Kosaki</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Prince G™</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>6955</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>ASHBORN™</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Nabila|Fortuners</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Ryujin Senju™</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>BlacKoreana O</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Meru™</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>683</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Signature</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Sesshomaru</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Flarekaze |Fortuners</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Raiden</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Breaker LITE</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>10032</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>+4917</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Kokyotosu</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Ary</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Morrissey</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>4986</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>14352</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+3706</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Rood</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>2951</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>6039</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>+522</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>1238</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-13 05:30:39
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -11138,11 +11138,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-13 13:00:13</t>
+          <t>Timestamp: 2026-08-13 13:30:36</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>14900</v>
+        <v>342</v>
       </c>
     </row>
     <row r="3">
@@ -11244,11 +11244,11 @@
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>3452</v>
+        <v>3560</v>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>+1944</t>
+          <t>+2052</t>
         </is>
       </c>
     </row>
@@ -11814,11 +11814,11 @@
         </is>
       </c>
       <c r="B47" s="3" t="n">
-        <v>10032</v>
+        <v>10140</v>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>+4917</t>
+          <t>+5025</t>
         </is>
       </c>
     </row>
@@ -11874,11 +11874,11 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>14352</v>
+        <v>14478</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+3706</t>
+          <t>+3832</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-13 05:55:39
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -11138,11 +11138,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-13 13:30:36</t>
+          <t>Timestamp: 2026-08-13 13:55:38</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>342</v>
+        <v>648</v>
       </c>
     </row>
     <row r="3">
@@ -11244,11 +11244,11 @@
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>3560</v>
+        <v>3668</v>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>+2052</t>
+          <t>+2160</t>
         </is>
       </c>
     </row>
@@ -11814,11 +11814,11 @@
         </is>
       </c>
       <c r="B47" s="3" t="n">
-        <v>10140</v>
+        <v>10248</v>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>+5025</t>
+          <t>+5133</t>
         </is>
       </c>
     </row>
@@ -11874,11 +11874,11 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>14478</v>
+        <v>14568</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+3832</t>
+          <t>+3922</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-14 05:00:13
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -27,6 +27,7 @@
     <sheet name="2026-08-11" sheetId="18" state="visible" r:id="rId18"/>
     <sheet name="2026-08-12" sheetId="19" state="visible" r:id="rId19"/>
     <sheet name="2026-08-13" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="2026-08-14" sheetId="21" state="visible" r:id="rId21"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -11996,6 +11997,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105) | S63</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-14 13:00:12</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>13759</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>NAOR</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>1956</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>4532</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>+864</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>£_Darkz_£</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>DangerousEX</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Xylota x [NvL]</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>8850</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>+2456</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>258</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>MATHEMATRICK</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Tobi</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Kosaki</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Prince G™</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>6955</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>ASHBORN™</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Nabila|Fortuners</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Ryujin Senju™</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>BlacKoreana O</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Meru™</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>683</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Signature</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Sesshomaru</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>+18</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Flarekaze |Fortuners</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Raiden</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Breaker LITE</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>12357</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>+2109</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Kokyotosu</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Arya</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Morrissey</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>6805</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>+1819</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>19297</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+4729</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>595</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>+576</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Rood</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>2951</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>6039</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>1778</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>+540</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-14 05:30:27
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -12027,11 +12027,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-14 13:00:12</t>
+          <t>Timestamp: 2026-08-14 13:30:27</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>13759</v>
+        <v>972</v>
       </c>
     </row>
     <row r="3">
@@ -12703,11 +12703,11 @@
         </is>
       </c>
       <c r="B47" s="3" t="n">
-        <v>12357</v>
+        <v>12465</v>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>+2109</t>
+          <t>+2217</t>
         </is>
       </c>
     </row>
@@ -12748,11 +12748,11 @@
         </is>
       </c>
       <c r="B50" s="3" t="n">
-        <v>6805</v>
+        <v>7021</v>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>+1819</t>
+          <t>+2035</t>
         </is>
       </c>
     </row>
@@ -12763,11 +12763,11 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>19297</v>
+        <v>19405</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+4729</t>
+          <t>+4837</t>
         </is>
       </c>
     </row>
@@ -12823,11 +12823,11 @@
         </is>
       </c>
       <c r="B55" s="3" t="n">
-        <v>2951</v>
+        <v>3491</v>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+540</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-14 05:53:59
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -12027,11 +12027,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-14 13:30:27</t>
+          <t>Timestamp: 2026-08-14 13:53:58</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>972</v>
+        <v>1188</v>
       </c>
     </row>
     <row r="3">
@@ -12703,11 +12703,11 @@
         </is>
       </c>
       <c r="B47" s="3" t="n">
-        <v>12465</v>
+        <v>12573</v>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>+2217</t>
+          <t>+2325</t>
         </is>
       </c>
     </row>
@@ -12763,11 +12763,11 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>19405</v>
+        <v>19513</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+4837</t>
+          <t>+4945</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-15 05:00:13
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -28,6 +28,7 @@
     <sheet name="2026-08-12" sheetId="19" state="visible" r:id="rId19"/>
     <sheet name="2026-08-13" sheetId="20" state="visible" r:id="rId20"/>
     <sheet name="2026-08-14" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="2026-08-15" sheetId="22" state="visible" r:id="rId22"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -12885,6 +12886,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105) | S63</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-15 13:00:12</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>19380</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>NAOR</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>1956</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>4532</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>£_Darkz_£</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>DangerousEX</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Xylota x [NvL]</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>8850</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>258</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>MATHEMATRICK</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Tobi</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>KOSAKI</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Prince G™</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>6955</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>ASHBORN™</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Nabila|Fortuners</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Ryujin Senju™</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>1296</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>+1296</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>BlacKoreana O</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>MERU™</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>2087</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>+1404</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Signature</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Sesshomaru</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Flarekaze |Fortuners</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Raiden</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Breaker LITE</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>15757</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>+3184</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Kokyotosu</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Arya</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Morrissey</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>9541</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>+2520</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>24396</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+4883</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>595</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Rood</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>8306</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+4815</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>6039</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>1868</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>+90</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-15 05:21:57
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -12916,11 +12916,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-15 13:00:12</t>
+          <t>Timestamp: 2026-08-15 13:21:56</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>19380</v>
+        <v>3348</v>
       </c>
     </row>
     <row r="3">
@@ -13337,11 +13337,11 @@
         </is>
       </c>
       <c r="B30" s="3" t="n">
-        <v>1296</v>
+        <v>2376</v>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>+1296</t>
+          <t>+2376</t>
         </is>
       </c>
     </row>
@@ -13397,11 +13397,11 @@
         </is>
       </c>
       <c r="B34" s="3" t="n">
-        <v>2087</v>
+        <v>3167</v>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>+1404</t>
+          <t>+2484</t>
         </is>
       </c>
     </row>
@@ -13637,11 +13637,11 @@
         </is>
       </c>
       <c r="B50" s="3" t="n">
-        <v>9541</v>
+        <v>10585</v>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>+2520</t>
+          <t>+3564</t>
         </is>
       </c>
     </row>
@@ -13652,11 +13652,11 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>24396</v>
+        <v>24612</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+4883</t>
+          <t>+5099</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-16 05:00:13
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -29,6 +29,7 @@
     <sheet name="2026-08-13" sheetId="20" state="visible" r:id="rId20"/>
     <sheet name="2026-08-14" sheetId="21" state="visible" r:id="rId21"/>
     <sheet name="2026-08-15" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="2026-08-16" sheetId="23" state="visible" r:id="rId23"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -13774,6 +13775,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105) | S63</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-16 13:00:12</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>50770</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>NAOR</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>1956</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>324</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>+288</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>4532</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>£_Darkz_£</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>DangerousEX</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Xylota x [NvL]</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>8850</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>258</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>MATHEMATRICK</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Tobi</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>KOSAKI</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>PRINCE G™</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>6955</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>ASHBORN™</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Nabila|Fortuners</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Izx Infernity</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>5692</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>+3316</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>BlacKoreana O</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>MERU™</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>11235</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>+8068</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Signature</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Sesshomaru</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Flarekaze |Fortuners</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Raiden</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Breaker LITE</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>24304</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>+8547</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Kokyotosu</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Arya</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Morrissey</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>15845</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>+5260</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>34554</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+9942</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>669</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>+74</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Rood</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>2160</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>+2160</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>18073</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+9767</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>6039</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>1868</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-16 05:24:49
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -13805,11 +13805,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-16 13:00:12</t>
+          <t>Timestamp: 2026-08-16 13:24:48</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>50770</v>
+        <v>216</v>
       </c>
     </row>
     <row r="3">
@@ -14541,11 +14541,11 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>34554</v>
+        <v>34770</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+9942</t>
+          <t>+10158</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-16 05:53:00
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -13805,11 +13805,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-16 13:30:30</t>
+          <t>Timestamp: 2026-08-16 13:52:59</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>216</v>
+        <v>397</v>
       </c>
     </row>
     <row r="3">
@@ -14541,11 +14541,11 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>34770</v>
+        <v>34951</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+10158</t>
+          <t>+10339</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-17 05:00:13
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -30,6 +30,7 @@
     <sheet name="2026-08-14" sheetId="21" state="visible" r:id="rId21"/>
     <sheet name="2026-08-15" sheetId="22" state="visible" r:id="rId22"/>
     <sheet name="2026-08-16" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="2026-08-17" sheetId="24" state="visible" r:id="rId24"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -14663,6 +14664,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105) | S63</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-17 13:00:12</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>37091</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>NAOR</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>1956</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>504</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>+180</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>4532</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>£_Darkz_£</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>DangerousEX</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Xylota x [NvL]</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>8850</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>258</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>MATHEMATRICK</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Tobi</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>KOSAKI</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>PRINCE G™</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>6955</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>ASHBORN™</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Nabila|Fortuners</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Izx Infernity</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>7852</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>+2160</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>BlacKoreana O</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>MERU™</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>18188</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>+6953</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Signature</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Sesshomaru</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Flarekaze |Fortuners</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Raiden</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Breaker LITE</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>29488</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>+5184</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Kokyotosu</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Arya</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Morrissey</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>20309</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>+4464</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>44747</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+9796</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>669</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Rood</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>3205</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>+1045</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>24985</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+6912</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>6039</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>1868</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-17 05:30:30
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -14694,11 +14694,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-17 13:00:12</t>
+          <t>Timestamp: 2026-08-17 13:30:29</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>37091</v>
+        <v>720</v>
       </c>
     </row>
     <row r="3">
@@ -15415,11 +15415,11 @@
         </is>
       </c>
       <c r="B50" s="3" t="n">
-        <v>20309</v>
+        <v>20849</v>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>+4464</t>
+          <t>+5004</t>
         </is>
       </c>
     </row>
@@ -15430,11 +15430,11 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>44747</v>
+        <v>44855</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+9796</t>
+          <t>+9904</t>
         </is>
       </c>
     </row>
@@ -15535,11 +15535,11 @@
         </is>
       </c>
       <c r="B58" s="3" t="n">
-        <v>1868</v>
+        <v>1940</v>
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+72</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-18 05:00:14
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -31,6 +31,7 @@
     <sheet name="2026-08-15" sheetId="22" state="visible" r:id="rId22"/>
     <sheet name="2026-08-16" sheetId="23" state="visible" r:id="rId23"/>
     <sheet name="2026-08-17" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="2026-08-18" sheetId="25" state="visible" r:id="rId25"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -15552,6 +15553,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105) | S63</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-18 13:00:13</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>16075</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>NAOR</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>2496</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>+540</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>612</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>+108</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>4532</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>£_Darkz_£</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>DangerousEX</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Xylota x [NvL]</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>8850</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>258</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>MATHEMATRICK</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Tobi</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>KOSAKI</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>PRINCE G™</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>6955</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>ASHBORN™</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Nabila|Fortuners</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Izx Infernity</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>7852</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>BlacKoreana O</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>MERU™</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>18188</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Signature</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Sesshomaru</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Flarekaze |Fortuners</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Raiden</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Breaker LITE</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>32358</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>+2870</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Kokyotosu</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Arya</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Morrissey</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>23801</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>+2952</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>49914</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+5059</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>669</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Rood</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>5223</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>+2018</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>26793</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+1808</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>6039</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>1940</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-18 05:25:12
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -15583,11 +15583,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-18 13:00:13</t>
+          <t>Timestamp: 2026-08-18 13:25:11</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>16075</v>
+        <v>108</v>
       </c>
     </row>
     <row r="3">
@@ -16319,11 +16319,11 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>49914</v>
+        <v>50022</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+5059</t>
+          <t>+5167</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-18 05:54:19
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -15583,11 +15583,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-18 13:30:29</t>
+          <t>Timestamp: 2026-08-18 13:54:18</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>108</v>
+        <v>540</v>
       </c>
     </row>
     <row r="3">
@@ -16319,11 +16319,11 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>50022</v>
+        <v>50130</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+5167</t>
+          <t>+5275</t>
         </is>
       </c>
     </row>
@@ -16379,11 +16379,11 @@
         </is>
       </c>
       <c r="B55" s="3" t="n">
-        <v>26793</v>
+        <v>27117</v>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>+1808</t>
+          <t>+2132</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-19 05:00:11
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -32,6 +32,7 @@
     <sheet name="2026-08-16" sheetId="23" state="visible" r:id="rId23"/>
     <sheet name="2026-08-17" sheetId="24" state="visible" r:id="rId24"/>
     <sheet name="2026-08-18" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="2026-08-19" sheetId="26" state="visible" r:id="rId26"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16441,6 +16442,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105) | S63</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-19 13:00:10</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>16759</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>NAOR</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>2496</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>612</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>4532</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>£_Darkz_£</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>DangerousEX</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Xylota x [NvL]</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>8850</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>258</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>MATHEMATRICK</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Tobi</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>KOSAKI</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>PRINCE G™</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>6955</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>ASHBORN™</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Nabila|Fortuners</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>1080</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>+1080</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Izx Infernity</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>7852</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>BlacKoreana O</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>MERU™</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>18188</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Signature</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Sesshomaru</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Flarekaze |Fortuners</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Raiden</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Breaker LITE</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>36013</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>+3655</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Kokyotosu</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Arya</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Morrissey</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>24899</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>+1098</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>55098</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+4968</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>777</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>+108</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Rood</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>5241</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>+18</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>31869</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+4752</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>6039</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>2480</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>+540</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-19 05:26:38
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -16472,11 +16472,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-19 13:00:10</t>
+          <t>Timestamp: 2026-08-19 13:26:37</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>16759</v>
+        <v>378</v>
       </c>
     </row>
     <row r="3">
@@ -17193,11 +17193,11 @@
         </is>
       </c>
       <c r="B50" s="3" t="n">
-        <v>24899</v>
+        <v>25169</v>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>+1098</t>
+          <t>+1368</t>
         </is>
       </c>
     </row>
@@ -17208,11 +17208,11 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>55098</v>
+        <v>55206</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+4968</t>
+          <t>+5076</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-19 05:55:35
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -16472,11 +16472,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-19 13:30:26</t>
+          <t>Timestamp: 2026-08-19 13:55:33</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>378</v>
+        <v>918</v>
       </c>
     </row>
     <row r="3">
@@ -17148,11 +17148,11 @@
         </is>
       </c>
       <c r="B47" s="3" t="n">
-        <v>36013</v>
+        <v>36229</v>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>+3655</t>
+          <t>+3871</t>
         </is>
       </c>
     </row>
@@ -17208,11 +17208,11 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>55206</v>
+        <v>55314</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+5076</t>
+          <t>+5184</t>
         </is>
       </c>
     </row>
@@ -17268,11 +17268,11 @@
         </is>
       </c>
       <c r="B55" s="3" t="n">
-        <v>31869</v>
+        <v>32085</v>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>+4752</t>
+          <t>+4968</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-20 05:00:11
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -33,6 +33,7 @@
     <sheet name="2026-08-17" sheetId="24" state="visible" r:id="rId24"/>
     <sheet name="2026-08-18" sheetId="25" state="visible" r:id="rId25"/>
     <sheet name="2026-08-19" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="2026-08-20" sheetId="27" state="visible" r:id="rId27"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17330,6 +17331,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105) | S63</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-20 13:00:11</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>11840</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Spirit</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>NAOR</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>2496</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>630</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>+18</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>4532</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>£_Darkz_£</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>DangerousEX</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Xylota x [NvL]</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>8850</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>258</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>MATHEMATRICK</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Tobi</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>KOSAKI</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>PRINCE G™</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>6955</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>ASHBORN™</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Nabila|Fortuners</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>1080</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Izx Infernity</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>7852</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>BlacKoreana O</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>540</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+540</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>MERU™</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>18188</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Signature</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Sesshomaru</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Flarekaze |Fortuners</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Raiden</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Breaker LITE</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>38463</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>+2234</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>TYSM for Market Devs</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Arya</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Morrissey</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>25169</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>59874</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+4560</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>777</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Rood</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>5241</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>35655</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+3570</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>6039</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>2480</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-20 05:27:18
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -17361,11 +17361,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-20 13:00:11</t>
+          <t>Timestamp: 2026-08-20 13:27:17</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>11840</v>
+        <v>216</v>
       </c>
     </row>
     <row r="3">
@@ -18097,11 +18097,11 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>59874</v>
+        <v>59982</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+4560</t>
+          <t>+4668</t>
         </is>
       </c>
     </row>
@@ -18157,11 +18157,11 @@
         </is>
       </c>
       <c r="B55" s="3" t="n">
-        <v>35655</v>
+        <v>35763</v>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>+3570</t>
+          <t>+3678</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-20 05:56:39
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -17361,11 +17361,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-20 13:30:24</t>
+          <t>Timestamp: 2026-08-20 13:56:38</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>216</v>
+        <v>330</v>
       </c>
     </row>
     <row r="3">
@@ -18097,11 +18097,11 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>59982</v>
+        <v>59988</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+4668</t>
+          <t>+4674</t>
         </is>
       </c>
     </row>
@@ -18157,11 +18157,11 @@
         </is>
       </c>
       <c r="B55" s="3" t="n">
-        <v>35763</v>
+        <v>35871</v>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>+3678</t>
+          <t>+3786</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-21 05:00:12
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -34,6 +34,7 @@
     <sheet name="2026-08-18" sheetId="25" state="visible" r:id="rId25"/>
     <sheet name="2026-08-19" sheetId="26" state="visible" r:id="rId26"/>
     <sheet name="2026-08-20" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="2026-08-21" sheetId="28" state="visible" r:id="rId28"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18219,6 +18220,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105) | S63</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-21 13:00:12</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>28362</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>$ p i r i t</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>108</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>NAOR</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>2496</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>630</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>6800</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>+2268</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>£_Darkz_£</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>DangerousEX</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Xylota x [NvL]</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>8850</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>540</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>+540</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>258</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>BlackObito™</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Tobi</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>KOSAKI</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>PRINCE G™</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>9871</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>+2916</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>ASHBORN™</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Nabila|Fortuners</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>1080</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Izx Infernity</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>9256</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>+1404</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>BlacKoreana O</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>4320</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+3780</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>MERU™</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>19484</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>+1296</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Signature</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Sesshomaru</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Flarekaze |Fortuners</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Raiden</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Breaker LITE</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>40839</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>+2376</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>TYSM for Market Devs</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Arya</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Morrissey †</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>25710</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>64956</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+4968</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>777</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Rood</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>5241</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>40646</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+4775</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>9063</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>+3024</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>2516</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>+36</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-21 05:28:49
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -18250,11 +18250,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-21 13:00:12</t>
+          <t>Timestamp: 2026-08-21 13:28:48</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>28362</v>
+        <v>864</v>
       </c>
     </row>
     <row r="3">
@@ -18356,11 +18356,11 @@
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>6800</v>
+        <v>6908</v>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>+2268</t>
+          <t>+2376</t>
         </is>
       </c>
     </row>
@@ -18581,11 +18581,11 @@
         </is>
       </c>
       <c r="B24" s="3" t="n">
-        <v>9871</v>
+        <v>9979</v>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>+2916</t>
+          <t>+3024</t>
         </is>
       </c>
     </row>
@@ -18671,11 +18671,11 @@
         </is>
       </c>
       <c r="B30" s="3" t="n">
-        <v>9256</v>
+        <v>9364</v>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>+1404</t>
+          <t>+1512</t>
         </is>
       </c>
     </row>
@@ -18686,11 +18686,11 @@
         </is>
       </c>
       <c r="B31" s="3" t="n">
-        <v>4320</v>
+        <v>4536</v>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>+3780</t>
+          <t>+3996</t>
         </is>
       </c>
     </row>
@@ -18731,11 +18731,11 @@
         </is>
       </c>
       <c r="B34" s="3" t="n">
-        <v>19484</v>
+        <v>19592</v>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>+1296</t>
+          <t>+1404</t>
         </is>
       </c>
     </row>
@@ -18986,11 +18986,11 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>64956</v>
+        <v>65064</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+4968</t>
+          <t>+5076</t>
         </is>
       </c>
     </row>
@@ -19076,11 +19076,11 @@
         </is>
       </c>
       <c r="B57" s="3" t="n">
-        <v>9063</v>
+        <v>9171</v>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>+3024</t>
+          <t>+3132</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-21 05:30:30
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -18250,11 +18250,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-21 13:28:48</t>
+          <t>Timestamp: 2026-08-21 13:30:29</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>864</v>
+        <v>865</v>
       </c>
     </row>
     <row r="3">
@@ -18731,11 +18731,11 @@
         </is>
       </c>
       <c r="B34" s="3" t="n">
-        <v>19592</v>
+        <v>19593</v>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>+1404</t>
+          <t>+1405</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-21 05:58:57
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -18250,11 +18250,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-21 13:30:29</t>
+          <t>Timestamp: 2026-08-21 13:58:55</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>865</v>
+        <v>1734</v>
       </c>
     </row>
     <row r="3">
@@ -18356,11 +18356,11 @@
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>6908</v>
+        <v>7016</v>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>+2376</t>
+          <t>+2484</t>
         </is>
       </c>
     </row>
@@ -18581,11 +18581,11 @@
         </is>
       </c>
       <c r="B24" s="3" t="n">
-        <v>9979</v>
+        <v>10087</v>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>+3024</t>
+          <t>+3132</t>
         </is>
       </c>
     </row>
@@ -18671,11 +18671,11 @@
         </is>
       </c>
       <c r="B30" s="3" t="n">
-        <v>9364</v>
+        <v>9472</v>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>+1512</t>
+          <t>+1620</t>
         </is>
       </c>
     </row>
@@ -18686,11 +18686,11 @@
         </is>
       </c>
       <c r="B31" s="3" t="n">
-        <v>4536</v>
+        <v>4644</v>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>+3996</t>
+          <t>+4104</t>
         </is>
       </c>
     </row>
@@ -18731,11 +18731,11 @@
         </is>
       </c>
       <c r="B34" s="3" t="n">
-        <v>19593</v>
+        <v>19598</v>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>+1405</t>
+          <t>+1410</t>
         </is>
       </c>
     </row>
@@ -18986,11 +18986,11 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>65064</v>
+        <v>65172</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+5076</t>
+          <t>+5184</t>
         </is>
       </c>
     </row>
@@ -19046,11 +19046,11 @@
         </is>
       </c>
       <c r="B55" s="3" t="n">
-        <v>40646</v>
+        <v>40970</v>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>+4775</t>
+          <t>+5099</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-22 05:00:12
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -35,6 +35,7 @@
     <sheet name="2026-08-19" sheetId="26" state="visible" r:id="rId26"/>
     <sheet name="2026-08-20" sheetId="27" state="visible" r:id="rId27"/>
     <sheet name="2026-08-21" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="2026-08-22" sheetId="29" state="visible" r:id="rId29"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19108,6 +19109,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105) | S63</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-22 13:00:11</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>36086</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>$ p i r i t</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>108</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>NAOR</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>2496</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>666</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>+36</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>10688</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>+3672</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>£_Darkz_£</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>AstreaEX</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>ReinEX</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>8850</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>540</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>258</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Izuna</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Tobi</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>KOSAKI</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>PRINCE G™</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>13759</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>+3672</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>MATHEMATRICK</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Nabila|Fortuners</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>1603</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>+523</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Ryujin Senju™</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>12496</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>+3024</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>ZenithEX</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>8066</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>MERU™</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>LA NEGRA MATEA</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>22406</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Signature</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Sesshomaru</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Flarekaze |Fortuners</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Raiden</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>540</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>+540</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Breaker LITE</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>44943</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>+4104</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>TYSM for Market Devs</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Arya</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Sirius Kurogaeshi</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>25746</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>70140</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+4968</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>777</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Rood</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>5241</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>44231</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+3261</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>13457</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>+4286</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>2516</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-22 05:00:29
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -19139,11 +19139,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-22 13:00:11</t>
+          <t>Timestamp: 2026-08-22 13:00:27</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>36086</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
auto: snapshot 2026-08-22 05:30:27
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -19139,11 +19139,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-22 13:00:27</t>
+          <t>Timestamp: 2026-08-22 13:30:25</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0</v>
+        <v>2055</v>
       </c>
     </row>
     <row r="3">
@@ -19245,11 +19245,11 @@
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>10688</v>
+        <v>10904</v>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>+3672</t>
+          <t>+3888</t>
         </is>
       </c>
     </row>
@@ -19560,11 +19560,11 @@
         </is>
       </c>
       <c r="B30" s="3" t="n">
-        <v>12496</v>
+        <v>12712</v>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>+3024</t>
+          <t>+3240</t>
         </is>
       </c>
     </row>
@@ -19575,7 +19575,7 @@
         </is>
       </c>
       <c r="B31" s="3" t="n">
-        <v>8066</v>
+        <v>9146</v>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
@@ -19620,7 +19620,7 @@
         </is>
       </c>
       <c r="B34" s="3" t="n">
-        <v>22406</v>
+        <v>22622</v>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
@@ -19856,7 +19856,7 @@
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
         <is>
-          <t>Sirius Kurogaeshi</t>
+          <t>Sirius Impera</t>
         </is>
       </c>
       <c r="B50" s="3" t="n">
@@ -19875,11 +19875,11 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>70140</v>
+        <v>70356</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+4968</t>
+          <t>+5184</t>
         </is>
       </c>
     </row>
@@ -19965,11 +19965,11 @@
         </is>
       </c>
       <c r="B57" s="3" t="n">
-        <v>13457</v>
+        <v>13568</v>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>+4286</t>
+          <t>+4397</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-22 05:34:23
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -19139,11 +19139,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-22 13:30:42</t>
+          <t>Timestamp: 2026-08-22 13:34:22</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>2055</v>
+        <v>2271</v>
       </c>
     </row>
     <row r="3">
@@ -19620,7 +19620,7 @@
         </is>
       </c>
       <c r="B34" s="3" t="n">
-        <v>22622</v>
+        <v>22838</v>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
@@ -19856,7 +19856,7 @@
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
         <is>
-          <t>Sirius Impera</t>
+          <t>Sirius Impéria</t>
         </is>
       </c>
       <c r="B50" s="3" t="n">

</xml_diff>

<commit_message>
auto: snapshot 2026-08-23 05:00:13
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -36,6 +36,7 @@
     <sheet name="2026-08-20" sheetId="27" state="visible" r:id="rId27"/>
     <sheet name="2026-08-21" sheetId="28" state="visible" r:id="rId28"/>
     <sheet name="2026-08-22" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="2026-08-23" sheetId="30" state="visible" r:id="rId30"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20885,6 +20886,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105) | S63</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-23 13:00:12</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>63825</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>$ p i r i t</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>432</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>+324</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>NAOR</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>2496</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>874</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>+208</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>SuhaibEX</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>14264</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>+3360</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>£_Darkz_£</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>AstreaEX</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>ReinEX</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>8850</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>540</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>258</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Izuna</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Tobi</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>KOSAKI</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>PRINCE G™</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>13759</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>MATHEMATRICK</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Nabila|Fortuners</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>1603</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Ryujin Senju™</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>21889</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>+9177</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>ZenithEX</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>9851</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+705</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>MERU™</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>LA NEGRA MATEA</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>31499</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>+8661</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Signature</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Sesshomaru</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>214</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>+204</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Flarekaze |Fortuners</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Raiden</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>1380</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>+840</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Breaker LITE</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>54045</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>+9102</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>TYSM for Market Devs</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>2666</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>+2666</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Arya</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Sirius</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>26586</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>79344</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+8988</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>777</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Rood</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>5241</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>51101</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+6870</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>840</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>+840</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>22337</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>+8769</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>2516</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-23 05:25:55
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -20916,11 +20916,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-23 13:00:12</t>
+          <t>Timestamp: 2026-08-23 13:25:54</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>63825</v>
+        <v>1848</v>
       </c>
     </row>
     <row r="3">
@@ -21022,11 +21022,11 @@
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>14264</v>
+        <v>14432</v>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>+3360</t>
+          <t>+3528</t>
         </is>
       </c>
     </row>
@@ -21337,11 +21337,11 @@
         </is>
       </c>
       <c r="B30" s="3" t="n">
-        <v>21889</v>
+        <v>22057</v>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>+9177</t>
+          <t>+9345</t>
         </is>
       </c>
     </row>
@@ -21397,11 +21397,11 @@
         </is>
       </c>
       <c r="B34" s="3" t="n">
-        <v>31499</v>
+        <v>31667</v>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>+8661</t>
+          <t>+8829</t>
         </is>
       </c>
     </row>
@@ -21592,11 +21592,11 @@
         </is>
       </c>
       <c r="B47" s="3" t="n">
-        <v>54045</v>
+        <v>54213</v>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>+9102</t>
+          <t>+9270</t>
         </is>
       </c>
     </row>
@@ -21637,7 +21637,7 @@
         </is>
       </c>
       <c r="B50" s="3" t="n">
-        <v>26586</v>
+        <v>27090</v>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
@@ -21652,11 +21652,11 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>79344</v>
+        <v>79512</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+8988</t>
+          <t>+9156</t>
         </is>
       </c>
     </row>
@@ -21712,11 +21712,11 @@
         </is>
       </c>
       <c r="B55" s="3" t="n">
-        <v>51101</v>
+        <v>51437</v>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>+6870</t>
+          <t>+7206</t>
         </is>
       </c>
     </row>
@@ -21742,11 +21742,11 @@
         </is>
       </c>
       <c r="B57" s="3" t="n">
-        <v>22337</v>
+        <v>22505</v>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>+8769</t>
+          <t>+8937</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-23 05:30:25
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -20916,11 +20916,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-23 13:25:54</t>
+          <t>Timestamp: 2026-08-23 13:30:24</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>1848</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="3">
@@ -21607,11 +21607,11 @@
         </is>
       </c>
       <c r="B48" s="3" t="n">
-        <v>2666</v>
+        <v>3366</v>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>+2666</t>
+          <t>+3366</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-23 05:54:18
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -20916,11 +20916,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-23 13:30:24</t>
+          <t>Timestamp: 2026-08-23 13:54:17</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>2548</v>
+        <v>3696</v>
       </c>
     </row>
     <row r="3">
@@ -21003,7 +21003,7 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>SuhaibEX</t>
+          <t>KosakiEX</t>
         </is>
       </c>
       <c r="B8" s="3" t="n">
@@ -21022,11 +21022,11 @@
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>14432</v>
+        <v>14600</v>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>+3528</t>
+          <t>+3696</t>
         </is>
       </c>
     </row>
@@ -21337,11 +21337,11 @@
         </is>
       </c>
       <c r="B30" s="3" t="n">
-        <v>22057</v>
+        <v>22225</v>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>+9345</t>
+          <t>+9513</t>
         </is>
       </c>
     </row>
@@ -21352,11 +21352,11 @@
         </is>
       </c>
       <c r="B31" s="3" t="n">
-        <v>9851</v>
+        <v>9935</v>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>+705</t>
+          <t>+789</t>
         </is>
       </c>
     </row>
@@ -21397,11 +21397,11 @@
         </is>
       </c>
       <c r="B34" s="3" t="n">
-        <v>31667</v>
+        <v>31835</v>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>+8829</t>
+          <t>+8997</t>
         </is>
       </c>
     </row>
@@ -21457,11 +21457,11 @@
         </is>
       </c>
       <c r="B38" s="3" t="n">
-        <v>214</v>
+        <v>242</v>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>+204</t>
+          <t>+232</t>
         </is>
       </c>
     </row>
@@ -21592,11 +21592,11 @@
         </is>
       </c>
       <c r="B47" s="3" t="n">
-        <v>54213</v>
+        <v>54381</v>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>+9270</t>
+          <t>+9438</t>
         </is>
       </c>
     </row>
@@ -21652,11 +21652,11 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>79512</v>
+        <v>79680</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+9156</t>
+          <t>+9324</t>
         </is>
       </c>
     </row>
@@ -21712,11 +21712,11 @@
         </is>
       </c>
       <c r="B55" s="3" t="n">
-        <v>51437</v>
+        <v>51605</v>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>+7206</t>
+          <t>+7374</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-23 05:56:12
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -20916,11 +20916,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-23 13:54:17</t>
+          <t>Timestamp: 2026-08-23 13:56:11</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>3696</v>
+        <v>4316</v>
       </c>
     </row>
     <row r="3">
@@ -21352,11 +21352,11 @@
         </is>
       </c>
       <c r="B31" s="3" t="n">
-        <v>9935</v>
+        <v>10583</v>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>+789</t>
+          <t>+1437</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-24 05:00:11
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -37,6 +37,7 @@
     <sheet name="2026-08-21" sheetId="28" state="visible" r:id="rId28"/>
     <sheet name="2026-08-22" sheetId="29" state="visible" r:id="rId29"/>
     <sheet name="2026-08-23" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet name="2026-08-24" sheetId="31" state="visible" r:id="rId31"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21774,6 +21775,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105) | S63</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-24 13:00:10</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>84239</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>$ p i r i t</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>432</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Harimukun</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>NAOR</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>2496</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>902</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>+28</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>18464</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>+3864</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>£_Darkz_£</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>AstreaEX</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>540</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>258</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Izuna</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>1680</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>+1680</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Tobi</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>KOSAKI</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>7107</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>+7107</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>PRINCE G™</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>4455</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>+4455</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>17185</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>+3426</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>MATHEMATRICK</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Nabila|Fortuners</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>1603</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Ryujin Senju™</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>25564</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>+3339</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>ZenithEX</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>12879</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+2296</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>MERU™</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>6780</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>+6780</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>PUCCA</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>36431</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Signature</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Sesshomaru</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>7149</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>+7149</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>242</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Flarekaze |Fortuners</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Raiden</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>2850</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>+1470</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Breaker LITE</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>57411</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>+3030</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>TYSM for Market Devs</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>5583</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>+2217</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Arya</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>5073</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>+5073</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Sirius</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>29050</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>+1960</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>87327</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+7647</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>777</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Rood</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>5241</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>57296</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+5691</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>840</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>29834</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>+7329</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>3302</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>+786</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-24 05:30:26
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -21805,11 +21805,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-24 13:00:10</t>
+          <t>Timestamp: 2026-08-24 13:30:25</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>84239</v>
+        <v>1114</v>
       </c>
     </row>
     <row r="3">
@@ -22076,11 +22076,11 @@
         </is>
       </c>
       <c r="B20" s="3" t="n">
-        <v>7107</v>
+        <v>7191</v>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>+7107</t>
+          <t>+7191</t>
         </is>
       </c>
     </row>
@@ -22091,11 +22091,11 @@
         </is>
       </c>
       <c r="B21" s="3" t="n">
-        <v>4455</v>
+        <v>4539</v>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>+4455</t>
+          <t>+4539</t>
         </is>
       </c>
     </row>
@@ -22271,11 +22271,11 @@
         </is>
       </c>
       <c r="B33" s="3" t="n">
-        <v>6780</v>
+        <v>6864</v>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>+6780</t>
+          <t>+6864</t>
         </is>
       </c>
     </row>
@@ -22331,11 +22331,11 @@
         </is>
       </c>
       <c r="B37" s="3" t="n">
-        <v>7149</v>
+        <v>7172</v>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>+7149</t>
+          <t>+7172</t>
         </is>
       </c>
     </row>
@@ -22481,11 +22481,11 @@
         </is>
       </c>
       <c r="B47" s="3" t="n">
-        <v>57411</v>
+        <v>57579</v>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>+3030</t>
+          <t>+3198</t>
         </is>
       </c>
     </row>
@@ -22511,11 +22511,11 @@
         </is>
       </c>
       <c r="B49" s="3" t="n">
-        <v>5073</v>
+        <v>5157</v>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>+5073</t>
+          <t>+5157</t>
         </is>
       </c>
     </row>
@@ -22541,11 +22541,11 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>87327</v>
+        <v>87411</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+7647</t>
+          <t>+7731</t>
         </is>
       </c>
     </row>
@@ -22601,11 +22601,11 @@
         </is>
       </c>
       <c r="B55" s="3" t="n">
-        <v>57296</v>
+        <v>57716</v>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>+5691</t>
+          <t>+6111</t>
         </is>
       </c>
     </row>
@@ -22631,11 +22631,11 @@
         </is>
       </c>
       <c r="B57" s="3" t="n">
-        <v>29834</v>
+        <v>29918</v>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>+7329</t>
+          <t>+7413</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-24 05:35:21
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -21805,11 +21805,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-24 13:30:25</t>
+          <t>Timestamp: 2026-08-24 13:35:20</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>1114</v>
+        <v>1284</v>
       </c>
     </row>
     <row r="3">
@@ -22091,11 +22091,11 @@
         </is>
       </c>
       <c r="B21" s="3" t="n">
-        <v>4539</v>
+        <v>4623</v>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>+4539</t>
+          <t>+4623</t>
         </is>
       </c>
     </row>
@@ -22331,11 +22331,11 @@
         </is>
       </c>
       <c r="B37" s="3" t="n">
-        <v>7172</v>
+        <v>7174</v>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>+7172</t>
+          <t>+7174</t>
         </is>
       </c>
     </row>
@@ -22541,11 +22541,11 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>87411</v>
+        <v>87495</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+7731</t>
+          <t>+7815</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-25 05:00:13
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -38,6 +38,7 @@
     <sheet name="2026-08-22" sheetId="29" state="visible" r:id="rId29"/>
     <sheet name="2026-08-23" sheetId="30" state="visible" r:id="rId30"/>
     <sheet name="2026-08-24" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet name="2026-08-25" sheetId="32" state="visible" r:id="rId32"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22663,6 +22664,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105) | S63</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-25 13:00:12</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>38759</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>$ p i r i t</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>432</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Harimukun</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>NAOR</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>2496</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>902</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>18464</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>£_Darkz_£</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>AstreaEX</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>2976</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>+2436</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>258</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Izuna</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>+350</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>1680</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Tobi</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>KOSAKI</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>11022</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>+3831</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>PRINCE G™</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>7206</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>+2583</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>17185</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>MATHEMATRICK</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Nabila|Fortuners</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>1603</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Ryujin Senju™</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>27160</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>+1596</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>ZenithEX</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>14139</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+1260</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>MERU™</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>10669</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>+3805</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>PUCCA</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>37943</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>+1512</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Signature</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Sesshomaru</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>9629</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>+2455</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>242</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>DeVana</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Raiden</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>2850</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Breaker LITE</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>61053</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>+3474</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>TYSM for Market Devs</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>5595</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>+12</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Arya</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>8865</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>+3708</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Sirius</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>29050</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>91281</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+3786</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>777</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Rood</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>5241</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>61023</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+3307</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>840</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>32858</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>+2940</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>3722</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>+420</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-25 05:28:03
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -22694,11 +22694,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-25 13:00:12</t>
+          <t>Timestamp: 2026-08-25 13:28:02</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>38759</v>
+        <v>588</v>
       </c>
     </row>
     <row r="3">
@@ -22860,11 +22860,11 @@
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>2976</v>
+        <v>3060</v>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>+2436</t>
+          <t>+2520</t>
         </is>
       </c>
     </row>
@@ -22965,11 +22965,11 @@
         </is>
       </c>
       <c r="B20" s="3" t="n">
-        <v>11022</v>
+        <v>11106</v>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>+3831</t>
+          <t>+3915</t>
         </is>
       </c>
     </row>
@@ -23115,11 +23115,11 @@
         </is>
       </c>
       <c r="B30" s="3" t="n">
-        <v>27160</v>
+        <v>27244</v>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>+1596</t>
+          <t>+1680</t>
         </is>
       </c>
     </row>
@@ -23175,11 +23175,11 @@
         </is>
       </c>
       <c r="B34" s="3" t="n">
-        <v>37943</v>
+        <v>38111</v>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>+1512</t>
+          <t>+1680</t>
         </is>
       </c>
     </row>
@@ -23220,11 +23220,11 @@
         </is>
       </c>
       <c r="B37" s="3" t="n">
-        <v>9629</v>
+        <v>9713</v>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>+2455</t>
+          <t>+2539</t>
         </is>
       </c>
     </row>
@@ -23430,11 +23430,11 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>91281</v>
+        <v>91365</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+3786</t>
+          <t>+3870</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-25 05:30:27
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -22694,11 +22694,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-25 13:28:02</t>
+          <t>Timestamp: 2026-08-25 13:30:27</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>588</v>
+        <v>648</v>
       </c>
     </row>
     <row r="3">
@@ -23520,11 +23520,11 @@
         </is>
       </c>
       <c r="B57" s="3" t="n">
-        <v>32858</v>
+        <v>32918</v>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>+2940</t>
+          <t>+3000</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-25 05:58:17
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -22694,11 +22694,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-25 13:30:27</t>
+          <t>Timestamp: 2026-08-25 13:58:16</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>648</v>
+        <v>1732</v>
       </c>
     </row>
     <row r="3">
@@ -22860,11 +22860,11 @@
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>3060</v>
+        <v>3144</v>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>+2520</t>
+          <t>+2604</t>
         </is>
       </c>
     </row>
@@ -22965,11 +22965,11 @@
         </is>
       </c>
       <c r="B20" s="3" t="n">
-        <v>11106</v>
+        <v>11190</v>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>+3915</t>
+          <t>+3999</t>
         </is>
       </c>
     </row>
@@ -22980,11 +22980,11 @@
         </is>
       </c>
       <c r="B21" s="3" t="n">
-        <v>7206</v>
+        <v>7374</v>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>+2583</t>
+          <t>+2751</t>
         </is>
       </c>
     </row>
@@ -23115,11 +23115,11 @@
         </is>
       </c>
       <c r="B30" s="3" t="n">
-        <v>27244</v>
+        <v>27328</v>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>+1680</t>
+          <t>+1764</t>
         </is>
       </c>
     </row>
@@ -23175,11 +23175,11 @@
         </is>
       </c>
       <c r="B34" s="3" t="n">
-        <v>38111</v>
+        <v>38195</v>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>+1680</t>
+          <t>+1764</t>
         </is>
       </c>
     </row>
@@ -23220,11 +23220,11 @@
         </is>
       </c>
       <c r="B37" s="3" t="n">
-        <v>9713</v>
+        <v>9784</v>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>+2539</t>
+          <t>+2610</t>
         </is>
       </c>
     </row>
@@ -23400,11 +23400,11 @@
         </is>
       </c>
       <c r="B49" s="3" t="n">
-        <v>8865</v>
+        <v>9117</v>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>+3708</t>
+          <t>+3960</t>
         </is>
       </c>
     </row>
@@ -23430,11 +23430,11 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>91365</v>
+        <v>91449</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+3870</t>
+          <t>+3954</t>
         </is>
       </c>
     </row>
@@ -23490,11 +23490,11 @@
         </is>
       </c>
       <c r="B55" s="3" t="n">
-        <v>61023</v>
+        <v>61191</v>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>+3307</t>
+          <t>+3475</t>
         </is>
       </c>
     </row>
@@ -23520,11 +23520,11 @@
         </is>
       </c>
       <c r="B57" s="3" t="n">
-        <v>32918</v>
+        <v>32923</v>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>+3000</t>
+          <t>+3005</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-26 05:00:12
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -39,6 +39,7 @@
     <sheet name="2026-08-23" sheetId="30" state="visible" r:id="rId30"/>
     <sheet name="2026-08-24" sheetId="31" state="visible" r:id="rId31"/>
     <sheet name="2026-08-25" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet name="2026-08-26" sheetId="33" state="visible" r:id="rId33"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23552,6 +23553,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105) | S63</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-26 13:00:11</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>55818</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>2618</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>+2618</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>$ p i r i t</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>432</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Harimukun</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>NAOR</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>2496</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>902</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>18464</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>£_Darkz_£</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>AstreaEX</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>10095</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>+6951</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>258</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Izuna</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>1680</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Tobi</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>KOSAKI</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>14963</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>+3773</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>PRINCE G™</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>11030</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>+3656</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>17185</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>MATHEMATRICK</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Nabila|Fortuners</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>1603</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Ryujin Senju™</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>30364</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>+3036</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>ZenithEX</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>16646</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+2507</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>MERU™</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>14279</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>+3610</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>40967</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Signature</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Sesshomaru</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>13245</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>+3461</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>242</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>3196</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>+3178</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>DeVana</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Raiden</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>2850</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Breaker LITE</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>64826</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>+3773</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>TYSM for Market Devs</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>5595</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Arya</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>12955</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>+3838</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Sirius</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>29050</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>95222</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+3773</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>777</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Rood</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>5241</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>64551</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+3360</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>840</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>36703</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>+3780</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>3722</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-26 05:30:26
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -23583,11 +23583,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-26 13:00:11</t>
+          <t>Timestamp: 2026-08-26 13:30:25</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>55818</v>
+        <v>1260</v>
       </c>
     </row>
     <row r="3">
@@ -23749,11 +23749,11 @@
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>10095</v>
+        <v>10179</v>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>+6951</t>
+          <t>+7035</t>
         </is>
       </c>
     </row>
@@ -23854,11 +23854,11 @@
         </is>
       </c>
       <c r="B20" s="3" t="n">
-        <v>14963</v>
+        <v>15047</v>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>+3773</t>
+          <t>+3857</t>
         </is>
       </c>
     </row>
@@ -23869,11 +23869,11 @@
         </is>
       </c>
       <c r="B21" s="3" t="n">
-        <v>11030</v>
+        <v>11114</v>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>+3656</t>
+          <t>+3740</t>
         </is>
       </c>
     </row>
@@ -23895,7 +23895,7 @@
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>NicolasRicko</t>
+          <t>ProfessorX ?</t>
         </is>
       </c>
       <c r="B23" s="3" t="n">
@@ -23903,18 +23903,18 @@
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>Izx Hatake Jr</t>
+          <t>NicolasRicko</t>
         </is>
       </c>
       <c r="B24" s="3" t="n">
-        <v>17185</v>
+        <v>0</v>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
@@ -23925,11 +23925,11 @@
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>MATHEMATRICK</t>
+          <t>Izx Hatake Jr</t>
         </is>
       </c>
       <c r="B25" s="3" t="n">
-        <v>0</v>
+        <v>17185</v>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
@@ -23940,7 +23940,7 @@
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>Nabila|Fortuners</t>
+          <t>MATHEMATRICK</t>
         </is>
       </c>
       <c r="B26" s="3" t="n">
@@ -23955,11 +23955,11 @@
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>~[AnbuDream]~</t>
+          <t>Nabila|Fortuners</t>
         </is>
       </c>
       <c r="B27" s="3" t="n">
-        <v>1603</v>
+        <v>0</v>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
@@ -23970,11 +23970,11 @@
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>Ryujin Senju™</t>
+          <t>~[AnbuDream]~</t>
         </is>
       </c>
       <c r="B28" s="3" t="n">
-        <v>0</v>
+        <v>1603</v>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
@@ -23985,7 +23985,7 @@
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Heisenberg </t>
+          <t>Ryujin Senju™</t>
         </is>
       </c>
       <c r="B29" s="3" t="n">
@@ -24000,97 +24000,97 @@
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>Tobirama Senju™</t>
+          <t xml:space="preserve">Heisenberg </t>
         </is>
       </c>
       <c r="B30" s="3" t="n">
-        <v>30364</v>
+        <v>0</v>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>+3036</t>
+          <t>0</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>ZenithEX</t>
+          <t>Tobirama Senju™</t>
         </is>
       </c>
       <c r="B31" s="3" t="n">
-        <v>16646</v>
+        <v>30364</v>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>+2507</t>
+          <t>+3036</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>§åñÐåïmårµ | Frtners</t>
+          <t>ZenithEX</t>
         </is>
       </c>
       <c r="B32" s="3" t="n">
-        <v>0</v>
+        <v>16646</v>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+2507</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>MERU™</t>
+          <t>§åñÐåïmårµ | Frtners</t>
         </is>
       </c>
       <c r="B33" s="3" t="n">
-        <v>14279</v>
+        <v>0</v>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>+3610</t>
+          <t>0</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>SNC | Vnzla Anbu |SN</t>
+          <t>MERU™</t>
         </is>
       </c>
       <c r="B34" s="3" t="n">
-        <v>40967</v>
+        <v>14363</v>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>+3694</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>SNC | Signature</t>
+          <t>SNC | Vnzla Anbu |SN</t>
         </is>
       </c>
       <c r="B35" s="3" t="n">
-        <v>0</v>
+        <v>41387</v>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>Fusion</t>
+          <t>SNC | Signature</t>
         </is>
       </c>
       <c r="B36" s="3" t="n">
@@ -24105,41 +24105,41 @@
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>Sesshomaru</t>
+          <t>Fusion</t>
         </is>
       </c>
       <c r="B37" s="3" t="n">
-        <v>13245</v>
+        <v>0</v>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>+3461</t>
+          <t>0</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t>KYO</t>
+          <t>Sesshomaru</t>
         </is>
       </c>
       <c r="B38" s="3" t="n">
-        <v>242</v>
+        <v>13329</v>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+3545</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nitro </t>
+          <t>KYO</t>
         </is>
       </c>
       <c r="B39" s="3" t="n">
-        <v>0</v>
+        <v>242</v>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
@@ -24150,37 +24150,37 @@
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
-          <t>SL41F3RT</t>
+          <t xml:space="preserve">Nitro </t>
         </is>
       </c>
       <c r="B40" s="3" t="n">
-        <v>3196</v>
+        <v>0</v>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>+3178</t>
+          <t>0</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>DeVana</t>
+          <t>SL41F3RT</t>
         </is>
       </c>
       <c r="B41" s="3" t="n">
-        <v>0</v>
+        <v>3196</v>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+3178</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
         <is>
-          <t>Raiden</t>
+          <t>DeVana</t>
         </is>
       </c>
       <c r="B42" s="3" t="n">
@@ -24195,11 +24195,11 @@
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
         <is>
-          <t>ShadowRavenX</t>
+          <t>Raiden</t>
         </is>
       </c>
       <c r="B43" s="3" t="n">
-        <v>2850</v>
+        <v>0</v>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
@@ -24210,11 +24210,11 @@
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
         <is>
-          <t>Aldrin</t>
+          <t>ShadowRavenX</t>
         </is>
       </c>
       <c r="B44" s="3" t="n">
-        <v>0</v>
+        <v>2850</v>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
@@ -24225,7 +24225,7 @@
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
         <is>
-          <t>SNC | TemperiTa</t>
+          <t>Aldrin</t>
         </is>
       </c>
       <c r="B45" s="3" t="n">
@@ -24240,7 +24240,7 @@
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
         <is>
-          <t>SmallDino</t>
+          <t>SNC | TemperiTa</t>
         </is>
       </c>
       <c r="B46" s="3" t="n">
@@ -24255,101 +24255,101 @@
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>Breaker LITE</t>
+          <t>SmallDino</t>
         </is>
       </c>
       <c r="B47" s="3" t="n">
-        <v>64826</v>
+        <v>0</v>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>+3773</t>
+          <t>0</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
         <is>
-          <t>TYSM for Market Devs</t>
+          <t>Breaker LITE</t>
         </is>
       </c>
       <c r="B48" s="3" t="n">
-        <v>5595</v>
+        <v>64994</v>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+3941</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t>Arya</t>
+          <t>TYSM for Market Devs</t>
         </is>
       </c>
       <c r="B49" s="3" t="n">
-        <v>12955</v>
+        <v>5595</v>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>+3838</t>
+          <t>0</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
         <is>
-          <t>Sirius</t>
+          <t>Arya</t>
         </is>
       </c>
       <c r="B50" s="3" t="n">
-        <v>29050</v>
+        <v>12955</v>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+3838</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>Jonny Brown</t>
+          <t>Sirius</t>
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>95222</v>
+        <v>29050</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>+3773</t>
+          <t>0</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
         <is>
-          <t>Knightwalker</t>
+          <t>Jonny Brown</t>
         </is>
       </c>
       <c r="B52" s="3" t="n">
-        <v>0</v>
+        <v>95306</v>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+3857</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">a fucking ninja </t>
+          <t>Knightwalker</t>
         </is>
       </c>
       <c r="B53" s="3" t="n">
-        <v>777</v>
+        <v>0</v>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
@@ -24360,11 +24360,11 @@
     <row r="54">
       <c r="A54" s="5" t="inlineStr">
         <is>
-          <t>Rood</t>
+          <t xml:space="preserve">a fucking ninja </t>
         </is>
       </c>
       <c r="B54" s="3" t="n">
-        <v>5241</v>
+        <v>777</v>
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
@@ -24409,11 +24409,11 @@
         </is>
       </c>
       <c r="B57" s="3" t="n">
-        <v>36703</v>
+        <v>36871</v>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>+3780</t>
+          <t>+3948</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-27 05:00:13
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -40,6 +40,7 @@
     <sheet name="2026-08-24" sheetId="31" state="visible" r:id="rId31"/>
     <sheet name="2026-08-25" sheetId="32" state="visible" r:id="rId32"/>
     <sheet name="2026-08-26" sheetId="33" state="visible" r:id="rId33"/>
+    <sheet name="2026-08-27" sheetId="34" state="visible" r:id="rId34"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -24441,6 +24442,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105) | S63</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-27 13:00:12</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>61244</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>3556</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>+938</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>$ p i r i t</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>895</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>+463</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Harimukun</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>420</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>+420</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>NAOR</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>2916</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>+420</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>902</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>2604</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>+2604</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>18464</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>£_Darkz_£</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>AstreaEX</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>14030</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>+3851</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>258</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Izuna</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>1680</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Tobi</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>KOSAKI</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>18904</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>+3857</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>PRINCE G™</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>14732</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>+3618</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>ProfessorX ?</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>2900</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>+2900</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>17185</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>MATHEMATRICK</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Nabila|Fortuners</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>1150</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>+1150</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>1603</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Ryujin Senju™</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>33633</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+3269</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>ZenithEX</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>19768</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>+3122</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>MERU™</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>18090</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>+3727</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>44411</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>+3024</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Signature</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>1092</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>+1092</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Sesshomaru</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>17186</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>+3857</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>242</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>3196</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>DeVana</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>1014</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>+1014</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Raiden</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>2850</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Breaker LITE</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>68838</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>+3844</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>TYSM for Market Devs</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>6015</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>+420</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Arya</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>17605</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>+4650</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Sirius</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>29050</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>98845</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>+3539</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>910</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>+910</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>791</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>+14</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>68046</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+3495</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>840</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>40657</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>+3786</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>3722</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-27 05:30:26
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -24472,11 +24472,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-27 13:00:12</t>
+          <t>Timestamp: 2026-08-27 13:30:25</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>61244</v>
+        <v>1796</v>
       </c>
     </row>
     <row r="3">
@@ -24578,11 +24578,11 @@
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>2604</v>
+        <v>2688</v>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>+2604</t>
+          <t>+2688</t>
         </is>
       </c>
     </row>
@@ -24638,11 +24638,11 @@
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>14030</v>
+        <v>14114</v>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>+3851</t>
+          <t>+3935</t>
         </is>
       </c>
     </row>
@@ -24743,11 +24743,11 @@
         </is>
       </c>
       <c r="B20" s="3" t="n">
-        <v>18904</v>
+        <v>18988</v>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>+3857</t>
+          <t>+3941</t>
         </is>
       </c>
     </row>
@@ -24848,11 +24848,11 @@
         </is>
       </c>
       <c r="B27" s="3" t="n">
-        <v>1150</v>
+        <v>1570</v>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>+1150</t>
+          <t>+1570</t>
         </is>
       </c>
     </row>
@@ -24908,11 +24908,11 @@
         </is>
       </c>
       <c r="B31" s="3" t="n">
-        <v>33633</v>
+        <v>33749</v>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>+3269</t>
+          <t>+3385</t>
         </is>
       </c>
     </row>
@@ -24923,11 +24923,11 @@
         </is>
       </c>
       <c r="B32" s="3" t="n">
-        <v>19768</v>
+        <v>19852</v>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>+3122</t>
+          <t>+3206</t>
         </is>
       </c>
     </row>
@@ -24953,11 +24953,11 @@
         </is>
       </c>
       <c r="B34" s="3" t="n">
-        <v>18090</v>
+        <v>18174</v>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>+3727</t>
+          <t>+3811</t>
         </is>
       </c>
     </row>
@@ -24968,11 +24968,11 @@
         </is>
       </c>
       <c r="B35" s="3" t="n">
-        <v>44411</v>
+        <v>44579</v>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>+3024</t>
+          <t>+3192</t>
         </is>
       </c>
     </row>
@@ -24998,11 +24998,11 @@
         </is>
       </c>
       <c r="B37" s="3" t="n">
-        <v>1092</v>
+        <v>1176</v>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>+1092</t>
+          <t>+1176</t>
         </is>
       </c>
     </row>
@@ -25013,11 +25013,11 @@
         </is>
       </c>
       <c r="B38" s="3" t="n">
-        <v>17186</v>
+        <v>17270</v>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>+3857</t>
+          <t>+3941</t>
         </is>
       </c>
     </row>
@@ -25178,11 +25178,11 @@
         </is>
       </c>
       <c r="B49" s="3" t="n">
-        <v>6015</v>
+        <v>6183</v>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>+420</t>
+          <t>+588</t>
         </is>
       </c>
     </row>
@@ -25193,11 +25193,11 @@
         </is>
       </c>
       <c r="B50" s="3" t="n">
-        <v>17605</v>
+        <v>17773</v>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>+4650</t>
+          <t>+4818</t>
         </is>
       </c>
     </row>
@@ -25223,11 +25223,11 @@
         </is>
       </c>
       <c r="B52" s="3" t="n">
-        <v>98845</v>
+        <v>98929</v>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>+3539</t>
+          <t>+3623</t>
         </is>
       </c>
     </row>
@@ -25298,11 +25298,11 @@
         </is>
       </c>
       <c r="B57" s="3" t="n">
-        <v>40657</v>
+        <v>40741</v>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>+3786</t>
+          <t>+3870</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-28 05:00:13
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -41,6 +41,7 @@
     <sheet name="2026-08-25" sheetId="32" state="visible" r:id="rId32"/>
     <sheet name="2026-08-26" sheetId="33" state="visible" r:id="rId33"/>
     <sheet name="2026-08-27" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet name="2026-08-28" sheetId="35" state="visible" r:id="rId35"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -25330,6 +25331,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105) | S63</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-28 13:00:12</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>51707</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>3556</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>$ p i r i t</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>895</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Harimukun</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>1344</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>+924</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>NAOR</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>3216</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>902</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>6036</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>+3348</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>18464</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>£_Darkz_£</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>AstreaEX</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>17542</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>+3428</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>258</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Izuna</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>1680</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Tobi</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>KOSAKI</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>21128</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>+2140</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>PRINCE G™</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>18236</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>+3504</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>ProfessorX ?</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>3508</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>+608</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>+20</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>17185</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>MATHEMATRICK</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Nabila|Fortuners</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>2562</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>+992</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>2323</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>+720</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Ryujin Senju™</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>36613</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+2864</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>ZenithEX</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>21472</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>+1620</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>MERU™</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>20814</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>+2640</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>47819</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>+3240</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Signature</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>4558</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>+3382</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Sesshomaru</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>20362</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>+3092</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>242</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>3196</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>DeVana</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>3209</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>+2195</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Raiden</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>2850</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Breaker LITE</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>72037</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>+3199</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>TYSM for Market Devs</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>6927</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>+744</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Arya</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>19188</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>+1415</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Sirius</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>29050</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>101388</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>+2459</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>910</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>791</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>71490</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+3444</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>840</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>44074</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>+3333</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>4022</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-28 05:05:27
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -25361,11 +25361,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-28 13:00:12</t>
+          <t>Timestamp: 2026-08-28 13:05:25</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>51707</v>
+        <v>31</v>
       </c>
     </row>
     <row r="3">
@@ -25857,11 +25857,11 @@
         </is>
       </c>
       <c r="B35" s="3" t="n">
-        <v>47819</v>
+        <v>47852</v>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>+3240</t>
+          <t>+3273</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-28 05:30:30
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -25361,11 +25361,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-28 13:05:25</t>
+          <t>Timestamp: 2026-08-28 13:30:29</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>31</v>
+        <v>571</v>
       </c>
     </row>
     <row r="3">
@@ -25467,11 +25467,11 @@
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>6036</v>
+        <v>6096</v>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>+3348</t>
+          <t>+3408</t>
         </is>
       </c>
     </row>
@@ -25527,11 +25527,11 @@
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>17542</v>
+        <v>17602</v>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>+3428</t>
+          <t>+3488</t>
         </is>
       </c>
     </row>
@@ -25632,11 +25632,11 @@
         </is>
       </c>
       <c r="B20" s="3" t="n">
-        <v>21128</v>
+        <v>21188</v>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>+2140</t>
+          <t>+2200</t>
         </is>
       </c>
     </row>
@@ -25647,11 +25647,11 @@
         </is>
       </c>
       <c r="B21" s="3" t="n">
-        <v>18236</v>
+        <v>18296</v>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>+3504</t>
+          <t>+3564</t>
         </is>
       </c>
     </row>
@@ -25812,11 +25812,11 @@
         </is>
       </c>
       <c r="B32" s="3" t="n">
-        <v>21472</v>
+        <v>21532</v>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>+1620</t>
+          <t>+1680</t>
         </is>
       </c>
     </row>
@@ -25842,11 +25842,11 @@
         </is>
       </c>
       <c r="B34" s="3" t="n">
-        <v>20814</v>
+        <v>20874</v>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>+2640</t>
+          <t>+2700</t>
         </is>
       </c>
     </row>
@@ -25887,11 +25887,11 @@
         </is>
       </c>
       <c r="B37" s="3" t="n">
-        <v>4558</v>
+        <v>4618</v>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>+3382</t>
+          <t>+3442</t>
         </is>
       </c>
     </row>
@@ -25902,11 +25902,11 @@
         </is>
       </c>
       <c r="B38" s="3" t="n">
-        <v>20362</v>
+        <v>20422</v>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>+3092</t>
+          <t>+3152</t>
         </is>
       </c>
     </row>
@@ -26187,11 +26187,11 @@
         </is>
       </c>
       <c r="B57" s="3" t="n">
-        <v>44074</v>
+        <v>44134</v>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>+3333</t>
+          <t>+3393</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-29 05:00:13
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -42,6 +42,7 @@
     <sheet name="2026-08-26" sheetId="33" state="visible" r:id="rId33"/>
     <sheet name="2026-08-27" sheetId="34" state="visible" r:id="rId34"/>
     <sheet name="2026-08-28" sheetId="35" state="visible" r:id="rId35"/>
+    <sheet name="2026-08-29" sheetId="36" state="visible" r:id="rId36"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -26219,6 +26220,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105) | S63</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-29 13:00:12</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>41721</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>3556</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>$ p i r i t</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>895</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Harimukun</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>1344</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>NAOR</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>3756</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>+540</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>2086</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>+1184</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>8916</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>+2820</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>18464</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>£_Darkz_£</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>AstreaEX</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>1782</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>+1782</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>18235</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>+633</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>258</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Izuna</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>2744</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>+1064</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Tobi</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>1047</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>+1047</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>KOSAKI</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>23201</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>+2013</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>PRINCE G™</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>21107</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>+2811</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>ProfessorX ?</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>3528</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>+20</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>17185</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>MATHEMATRICK</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Nabila|Fortuners</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>3282</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>+720</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>2623</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Ryujin Senju™</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>38284</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+1671</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>ZenithEX</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>22852</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>+1320</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>MERU™</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>22974</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>+2100</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>49892</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>+2040</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Signature</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>7420</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>+2802</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Sesshomaru</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>22522</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>+2100</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>252</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>+10</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>3196</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>FlareKaze</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>3749</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Raiden</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>3150</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Breaker LITE</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>74804</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>+2767</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>TYSM for Market Devs</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>7047</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>+120</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Arya</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>20988</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>+1800</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Sirius</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>29050</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>104282</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>+2894</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>910</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>791</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>74430</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+2940</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>840</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>46946</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>+2812</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>4022</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-29 05:30:28
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -26250,11 +26250,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-29 13:00:12</t>
+          <t>Timestamp: 2026-08-29 13:30:27</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>41721</v>
+        <v>1440</v>
       </c>
     </row>
     <row r="3">
@@ -26356,11 +26356,11 @@
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>8916</v>
+        <v>9036</v>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>+2820</t>
+          <t>+2940</t>
         </is>
       </c>
     </row>
@@ -26401,11 +26401,11 @@
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>1782</v>
+        <v>1902</v>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>+1782</t>
+          <t>+1902</t>
         </is>
       </c>
     </row>
@@ -26641,11 +26641,11 @@
         </is>
       </c>
       <c r="B28" s="3" t="n">
-        <v>2623</v>
+        <v>3223</v>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>+300</t>
+          <t>+900</t>
         </is>
       </c>
     </row>
@@ -26701,11 +26701,11 @@
         </is>
       </c>
       <c r="B32" s="3" t="n">
-        <v>22852</v>
+        <v>22972</v>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>+1320</t>
+          <t>+1440</t>
         </is>
       </c>
     </row>
@@ -26746,11 +26746,11 @@
         </is>
       </c>
       <c r="B35" s="3" t="n">
-        <v>49892</v>
+        <v>50012</v>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>+2040</t>
+          <t>+2160</t>
         </is>
       </c>
     </row>
@@ -26776,11 +26776,11 @@
         </is>
       </c>
       <c r="B37" s="3" t="n">
-        <v>7420</v>
+        <v>7540</v>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>+2802</t>
+          <t>+2922</t>
         </is>
       </c>
     </row>
@@ -27001,11 +27001,11 @@
         </is>
       </c>
       <c r="B52" s="3" t="n">
-        <v>104282</v>
+        <v>104402</v>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>+2894</t>
+          <t>+3014</t>
         </is>
       </c>
     </row>
@@ -27076,11 +27076,11 @@
         </is>
       </c>
       <c r="B57" s="3" t="n">
-        <v>46946</v>
+        <v>47066</v>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>+2812</t>
+          <t>+2932</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-30 05:00:11
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -43,6 +43,7 @@
     <sheet name="2026-08-27" sheetId="34" state="visible" r:id="rId34"/>
     <sheet name="2026-08-28" sheetId="35" state="visible" r:id="rId35"/>
     <sheet name="2026-08-29" sheetId="36" state="visible" r:id="rId36"/>
+    <sheet name="2026-08-30" sheetId="37" state="visible" r:id="rId37"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -27108,6 +27109,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105) | S63</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-30 13:00:10</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>40062</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>+36506</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>$ p i r i t</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>22393</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>+21498</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Harimukun</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>23727</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>+22383</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>NAOR</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>25921</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>+22165</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>23123</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>+21037</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>34467</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>+25431</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>35224</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>+16760</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>£_Darkz_£</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>23753</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>+23753</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>AstreaEX</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>28710</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>+26808</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>36279</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>+18044</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>22405</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>+22147</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Izuna</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>33630</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>+33630</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>37249</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>+36899</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>20248</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>+17504</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Tobi</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>36879</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>+35832</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>34947</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>+34947</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>KOSAKI</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>60702</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>+37501</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>PRINCE G™</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>44472</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>+23365</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>18710</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>+18710</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>ProfessorX ?</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>22626</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>+19098</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>21216</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>+21196</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>36659</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>+19474</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>MATHEMATRICK</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>17635</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>+17635</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Nabila|Fortuners</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>41258</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>+37976</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>25853</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>+22630</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Ryujin Senju™</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>15581</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>+15581</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>43903</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>+43903</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>66315</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+28031</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>ZenithEX</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>55737</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>+32765</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>44267</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>+44267</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>MERU™</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>43363</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>+20389</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>71765</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>+21753</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Signature</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>21025</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>+21025</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>32264</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>+24724</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Sesshomaru</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>50696</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>+28174</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>14208</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>+13956</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>35212</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>+35212</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>21387</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>+18191</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>FlareKaze</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>29775</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>+26026</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Raiden</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>20778</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>+20778</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>25701</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>+22551</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>20895</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>+20895</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>23544</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>+23544</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>22768</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>+22768</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Breaker LITE</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>104537</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>+29733</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>TYSM for Market Devs</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>30005</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>+22958</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Arya</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>55514</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>+34526</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Sirius</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>50380</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+21330</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>129766</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>+25364</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>24626</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>+23716</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>24305</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>+23514</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>101366</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+26936</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>24220</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>+23380</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>71119</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>+24053</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>21565</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>+17543</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-31 05:00:12
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -44,6 +44,7 @@
     <sheet name="2026-08-28" sheetId="35" state="visible" r:id="rId35"/>
     <sheet name="2026-08-29" sheetId="36" state="visible" r:id="rId36"/>
     <sheet name="2026-08-30" sheetId="37" state="visible" r:id="rId37"/>
+    <sheet name="2026-08-31" sheetId="38" state="visible" r:id="rId38"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -27997,6 +27998,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105) | S63</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-31 13:00:10</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>40062</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>$ p i r i t</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>22393</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Harimukun</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>23727</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>NAOR</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>25921</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>23123</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>34467</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>35224</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>£_Darkz_£</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>23753</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>AstreaEX</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>28710</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>36279</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>22405</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Izuna</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>33630</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>37249</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>20248</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Tobi</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>36879</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>34947</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>KOSAKI</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>60702</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>PRINCE G™</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>44472</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>18710</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>ProfessorX ?</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>22626</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>21216</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>36659</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>MATHEMATRICK</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>17635</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Nabila|Fortuners</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>41258</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>25853</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Ryujin Senju™</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>15581</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>43903</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>66315</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>ZenithEX</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>55737</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>44267</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>MERU™</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>43363</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>71765</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Signature</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>21025</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>32264</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Sesshomaru</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>50696</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>14208</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>35212</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>21387</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>FlareKaze</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>29775</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Raiden</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>20778</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>25701</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>20895</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>23544</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>22768</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Breaker LITE</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>104537</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>TYSM for Market Devs</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>30005</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Arya</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>55514</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Sirius</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>50380</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>129766</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>24626</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>24305</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>101366</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>24220</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>71119</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>21565</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-01 05:00:13
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -45,6 +45,7 @@
     <sheet name="2026-08-29" sheetId="36" state="visible" r:id="rId36"/>
     <sheet name="2026-08-30" sheetId="37" state="visible" r:id="rId37"/>
     <sheet name="2026-08-31" sheetId="38" state="visible" r:id="rId38"/>
+    <sheet name="2026-09-01" sheetId="39" state="visible" r:id="rId39"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -28886,6 +28887,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105) | S63</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-01 13:00:12</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>40062</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>$ p i r i t</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>22393</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Harimukun</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>23727</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>NAOR</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>25921</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>23123</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>34467</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>35224</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>£_Darkz_£</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>23753</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>AstreaEX</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>28710</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>36279</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>22405</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Izuna</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>33630</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>37249</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>20248</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Tobi</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>36879</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>34947</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>KOSAKI</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>60702</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>PRINCE G™</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>44472</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>18710</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>ProfessorX ?</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>22626</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>21216</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>36659</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>MATHEMATRICK</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>17635</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Nabila|Fortuners</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>41258</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>25853</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Ryujin Senju™</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>15581</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>43903</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>66315</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>ZenithEX</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>55737</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>44267</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>MERU™</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>43363</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>71765</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Signature</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>21025</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>32264</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Sesshomaru</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>50696</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>14208</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>35212</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>21387</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>FlareKaze</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>29775</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Raiden</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>20778</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>25701</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>20895</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>23544</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>22768</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Breaker LITE</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>104537</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>TYSM for Market Devs</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>30005</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Arya</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>55514</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Stüssy</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>50380</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>129766</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>24626</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>24305</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>101366</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>24220</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>71119</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>21565</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-02 05:00:15
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -46,6 +46,7 @@
     <sheet name="2026-08-30" sheetId="37" state="visible" r:id="rId37"/>
     <sheet name="2026-08-31" sheetId="38" state="visible" r:id="rId38"/>
     <sheet name="2026-09-01" sheetId="39" state="visible" r:id="rId39"/>
+    <sheet name="2026-09-02" sheetId="40" state="visible" r:id="rId40"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -30663,6 +30664,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105) | S64</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-02 13:00:12</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>$ p i r i t</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>219</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Harimukun</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>NAOR</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>£_Darkz_£</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>AstreaEX</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Izuna</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Tobi</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>KOSAKI</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>PRINCE G™</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>ProfessorX ?</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>MATHEMATRICK</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Nabila|Fortuners</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>443</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Ryujin Senju™</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>214</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>ZenithEX</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>MERU™</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>525</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Signature</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Sesshomaru</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Jembot Kriwil</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Raiden</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Breaker LITE</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>TYSM for Market Devs</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Arya</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Stüssy</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>252</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-02 05:30:29
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -30694,11 +30694,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-02 13:00:12</t>
+          <t>Timestamp: 2026-09-02 13:30:28</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0</v>
+        <v>44</v>
       </c>
     </row>
     <row r="3">
@@ -31130,7 +31130,7 @@
         </is>
       </c>
       <c r="B31" s="3" t="n">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
@@ -31430,7 +31430,7 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>252</v>
+        <v>293</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-03 05:00:13
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -47,6 +47,7 @@
     <sheet name="2026-08-31" sheetId="38" state="visible" r:id="rId38"/>
     <sheet name="2026-09-01" sheetId="39" state="visible" r:id="rId39"/>
     <sheet name="2026-09-02" sheetId="40" state="visible" r:id="rId40"/>
+    <sheet name="2026-09-03" sheetId="41" state="visible" r:id="rId41"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -31552,6 +31553,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105) | S64</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-03 13:00:12</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>16277</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>$ p i r i t</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>261</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>+42</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Harimukun</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>NAOR</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>420</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>+420</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>46</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>+46</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>£_Darkz_£</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>AstreaEX</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>+28</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>420</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>+420</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Izuna</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Tobi</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>KOSAKI</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>PRINCE G™</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>420</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>+420</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>ProfessorX ?</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>60</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>+56</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>MATHEMATRICK</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Nabila|Fortuners</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>831</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>+831</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>443</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Ryujin Senju™</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>2353</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+2136</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>ZenithEX</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>1802</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>+1802</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>MERU™</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>3001</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>+2476</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Signature</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Sesshomaru</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>+25</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>King Fortuners</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>738</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Raiden</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Breaker LITE</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>2790</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>+2790</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>TYSM for Market Devs</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Arya</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Stüssy</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>713</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+420</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>759</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>+759</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>370</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>+370</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>2328</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+2328</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>126</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>+126</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-03 05:30:30
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -31583,11 +31583,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-03 13:00:12</t>
+          <t>Timestamp: 2026-09-03 13:30:28</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>16277</v>
+        <v>168</v>
       </c>
     </row>
     <row r="3">
@@ -32079,11 +32079,11 @@
         </is>
       </c>
       <c r="B35" s="3" t="n">
-        <v>3001</v>
+        <v>3169</v>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>+2476</t>
+          <t>+2644</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-04 05:00:13
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -48,6 +48,7 @@
     <sheet name="2026-09-01" sheetId="39" state="visible" r:id="rId39"/>
     <sheet name="2026-09-02" sheetId="40" state="visible" r:id="rId40"/>
     <sheet name="2026-09-03" sheetId="41" state="visible" r:id="rId41"/>
+    <sheet name="2026-09-04" sheetId="42" state="visible" r:id="rId42"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -32441,6 +32442,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105) | S64</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-04 13:00:12</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>19327</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>$ p i r i t</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>261</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Harimukun</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>NAOR</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>840</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>+420</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>60</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>+14</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>£_Darkz_£</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>AstreaEX</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>420</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Izuna</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Tobi</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>KOSAKI</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>PRINCE G™</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>453</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>+33</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>ProfessorX ?</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>158</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>+98</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>MATHEMATRICK</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Nabila|Fortuners</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>831</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>443</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Ryujin Senju™</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>5641</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+3288</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>ZenithEX</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>3726</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>+1924</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>MERU™</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>5991</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>+2822</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Signature</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Sesshomaru</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>King Fortuners</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>738</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Raiden</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Breaker LITE</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>6354</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>+3564</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Kokyotosu</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Arya</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Stüssy</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>965</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+252</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>4609</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>+3850</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>370</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>5222</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+2894</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>126</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-04 05:28:06
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -32472,11 +32472,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-04 13:00:12</t>
+          <t>Timestamp: 2026-09-04 13:28:05</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>19327</v>
+        <v>420</v>
       </c>
     </row>
     <row r="3">
@@ -32908,11 +32908,11 @@
         </is>
       </c>
       <c r="B31" s="3" t="n">
-        <v>5641</v>
+        <v>5809</v>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>+3288</t>
+          <t>+3456</t>
         </is>
       </c>
     </row>
@@ -33163,11 +33163,11 @@
         </is>
       </c>
       <c r="B48" s="3" t="n">
-        <v>6354</v>
+        <v>6438</v>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>+3564</t>
+          <t>+3648</t>
         </is>
       </c>
     </row>
@@ -33223,11 +33223,11 @@
         </is>
       </c>
       <c r="B52" s="3" t="n">
-        <v>4609</v>
+        <v>4693</v>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>+3850</t>
+          <t>+3934</t>
         </is>
       </c>
     </row>
@@ -33268,11 +33268,11 @@
         </is>
       </c>
       <c r="B55" s="3" t="n">
-        <v>5222</v>
+        <v>5306</v>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>+2894</t>
+          <t>+2978</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-04 05:58:23
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -32472,11 +32472,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-04 13:30:29</t>
+          <t>Timestamp: 2026-09-04 13:58:22</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>420</v>
+        <v>504</v>
       </c>
     </row>
     <row r="3">
@@ -33223,11 +33223,11 @@
         </is>
       </c>
       <c r="B52" s="3" t="n">
-        <v>4693</v>
+        <v>4777</v>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>+3934</t>
+          <t>+4018</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-05 05:00:11
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -49,6 +49,7 @@
     <sheet name="2026-09-02" sheetId="40" state="visible" r:id="rId40"/>
     <sheet name="2026-09-03" sheetId="41" state="visible" r:id="rId41"/>
     <sheet name="2026-09-04" sheetId="42" state="visible" r:id="rId42"/>
+    <sheet name="2026-09-05" sheetId="43" state="visible" r:id="rId43"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -33330,6 +33331,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105) | S64</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-05 13:00:10</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>22902</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>$ p i r i t</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>261</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Harimukun</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>NAOR</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>1589</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>+749</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>74</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>+14</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>1008</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>+1008</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>£_Darkz_£</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>AstreaEX</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>820</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>+400</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Izuna</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Tobi</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>KOSAKI</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>PRINCE G™</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>453</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>ProfessorX ?</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>158</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>MATHEMATRICK</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Nabila|Fortuners</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>1671</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>+840</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>443</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Ryujin Senju™</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>9380</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+3571</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>ZenithEX</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>3726</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>MERU™</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>9892</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>+3901</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Signature</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Sesshomaru</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>King Fortuners</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>1203</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>+465</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Raiden</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>420</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>+420</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Breaker LITE</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>9836</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>+3398</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Kokyotosu</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Arya</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Stüssy</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>2143</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+1178</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>8459</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>+3682</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>370</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>8078</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+2772</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>126</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-05 05:30:25
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -33361,11 +33361,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-05 13:00:10</t>
+          <t>Timestamp: 2026-09-05 13:30:23</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>22902</v>
+        <v>423</v>
       </c>
     </row>
     <row r="3">
@@ -34112,11 +34112,11 @@
         </is>
       </c>
       <c r="B52" s="3" t="n">
-        <v>8459</v>
+        <v>8627</v>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>+3682</t>
+          <t>+3850</t>
         </is>
       </c>
     </row>
@@ -34157,11 +34157,11 @@
         </is>
       </c>
       <c r="B55" s="3" t="n">
-        <v>8078</v>
+        <v>8333</v>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>+2772</t>
+          <t>+3027</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-06 05:00:12
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -50,6 +50,7 @@
     <sheet name="2026-09-03" sheetId="41" state="visible" r:id="rId41"/>
     <sheet name="2026-09-04" sheetId="42" state="visible" r:id="rId42"/>
     <sheet name="2026-09-05" sheetId="43" state="visible" r:id="rId43"/>
+    <sheet name="2026-09-06" sheetId="44" state="visible" r:id="rId44"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -34219,6 +34220,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105) | S64</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-06 13:00:11</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>36157</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>$ p i r i t</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>261</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Harimukun</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>NAOR</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>2429</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>+840</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>102</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>+28</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>3528</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>+2520</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>£_Darkz_£</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>AstreaEX</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>820</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Izuna</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Tobi</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>KOSAKI</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>PRINCE G™</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>453</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>ProfessorX ?</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>410</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>+252</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>MATHEMATRICK</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Devia Ayu</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>2511</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>443</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Ryujin Senju™</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>16394</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+7014</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>ZenithEX</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>8631</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>+4905</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>MERU™</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>14608</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>+4716</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Signature</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Sesshomaru</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>King Fortuners</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>1203</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Raiden</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>420</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Breaker LITE</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>9836</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Kokyotosu</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Arya</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Stüssy</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>4777</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+2634</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>15814</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>+7187</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>370</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>+28</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>13103</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+4770</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>126</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-06 05:30:26
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -34250,11 +34250,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-06 13:00:11</t>
+          <t>Timestamp: 2026-09-06 13:30:25</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>36157</v>
+        <v>1512</v>
       </c>
     </row>
     <row r="3">
@@ -34686,11 +34686,11 @@
         </is>
       </c>
       <c r="B31" s="3" t="n">
-        <v>16394</v>
+        <v>17234</v>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>+7014</t>
+          <t>+7854</t>
         </is>
       </c>
     </row>
@@ -35001,11 +35001,11 @@
         </is>
       </c>
       <c r="B52" s="3" t="n">
-        <v>15814</v>
+        <v>16150</v>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>+7187</t>
+          <t>+7523</t>
         </is>
       </c>
     </row>
@@ -35046,11 +35046,11 @@
         </is>
       </c>
       <c r="B55" s="3" t="n">
-        <v>13103</v>
+        <v>13439</v>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>+4770</t>
+          <t>+5106</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-07 05:00:12
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -51,6 +51,7 @@
     <sheet name="2026-09-04" sheetId="42" state="visible" r:id="rId42"/>
     <sheet name="2026-09-05" sheetId="43" state="visible" r:id="rId43"/>
     <sheet name="2026-09-06" sheetId="44" state="visible" r:id="rId44"/>
+    <sheet name="2026-09-07" sheetId="45" state="visible" r:id="rId45"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -35108,6 +35109,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105) | S64</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-07 13:00:11</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>49705</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>$ p i r i t</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>289</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>+28</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Harimukun</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>NAOR</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>5151</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>+2722</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>130</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>+28</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>7056</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>+3528</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>£_Darkz_£</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>AstreaEX</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>820</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Izuna</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Tobi</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>KOSAKI</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>PRINCE G™</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>503</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>+50</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>ProfessorX ?</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>606</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>+196</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>MATHEMATRICK</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Devia Ayu</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>2511</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>443</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Ryujin Senju™</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>23093</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+5859</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>ZenithEX</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>13407</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>+4776</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>MERU™</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>21253</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>+6645</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Signature</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Sesshomaru</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>+28</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>King Fortuners</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>1203</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Raiden</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>420</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Breaker LITE</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>14078</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>+4242</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Kokyotosu</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>1008</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>+1008</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Arya</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Stüssy</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>5622</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+845</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>23992</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>+7842</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>370</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>20111</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+6672</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>3696</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>+3696</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>154</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>+28</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-07 05:30:26
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -35139,11 +35139,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-07 13:00:11</t>
+          <t>Timestamp: 2026-09-07 13:30:25</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>49705</v>
+        <v>291</v>
       </c>
     </row>
     <row r="3">
@@ -35575,11 +35575,11 @@
         </is>
       </c>
       <c r="B31" s="3" t="n">
-        <v>23093</v>
+        <v>23153</v>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>+5859</t>
+          <t>+5919</t>
         </is>
       </c>
     </row>
@@ -35635,11 +35635,11 @@
         </is>
       </c>
       <c r="B35" s="3" t="n">
-        <v>21253</v>
+        <v>21313</v>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>+6645</t>
+          <t>+6705</t>
         </is>
       </c>
     </row>
@@ -35830,11 +35830,11 @@
         </is>
       </c>
       <c r="B48" s="3" t="n">
-        <v>14078</v>
+        <v>14138</v>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>+4242</t>
+          <t>+4302</t>
         </is>
       </c>
     </row>
@@ -35890,11 +35890,11 @@
         </is>
       </c>
       <c r="B52" s="3" t="n">
-        <v>23992</v>
+        <v>24052</v>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>+7842</t>
+          <t>+7902</t>
         </is>
       </c>
     </row>
@@ -35935,11 +35935,11 @@
         </is>
       </c>
       <c r="B55" s="3" t="n">
-        <v>20111</v>
+        <v>20162</v>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>+6672</t>
+          <t>+6723</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-08 05:00:14
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -52,6 +52,7 @@
     <sheet name="2026-09-05" sheetId="43" state="visible" r:id="rId43"/>
     <sheet name="2026-09-06" sheetId="44" state="visible" r:id="rId44"/>
     <sheet name="2026-09-07" sheetId="45" state="visible" r:id="rId45"/>
+    <sheet name="2026-09-08" sheetId="46" state="visible" r:id="rId46"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -35997,6 +35998,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105) | S64</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-08 13:00:13</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>4020</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>$ p i r i t</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>359</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>+70</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Harimukun</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>NAOR</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>5832</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>+681</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>130</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>7226</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>+170</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>£_Darkz_£</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>AstreaEX</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>820</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Tobi</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>KOSAKI</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>PRINCE G™</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>503</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>ProfessorX ?</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>626</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>+20</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>MATHEMATRICK</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Devia Ayu</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>3126</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>+615</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>723</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>+280</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Ryujin Senju™</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>26052</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+2899</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>ZenithEX</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>14409</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>+1002</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>MERU™</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>23624</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>+2311</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Signature</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Sesshomaru</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>King Fortuners</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>1203</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Raiden</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>420</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Hail AangEX</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>15162</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Kokyotosu</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>2260</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>+1252</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Arya</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Stüssy</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>5622</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>26775</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>+2723</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>370</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>22248</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+2086</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>5399</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>+1703</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>184</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>+30</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-08 05:30:31
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -36028,11 +36028,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-08 13:00:13</t>
+          <t>Timestamp: 2026-09-08 13:30:29</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>4020</v>
+        <v>120</v>
       </c>
     </row>
     <row r="3">
@@ -36779,11 +36779,11 @@
         </is>
       </c>
       <c r="B52" s="3" t="n">
-        <v>26775</v>
+        <v>26835</v>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>+2723</t>
+          <t>+2783</t>
         </is>
       </c>
     </row>
@@ -36854,11 +36854,11 @@
         </is>
       </c>
       <c r="B57" s="3" t="n">
-        <v>5399</v>
+        <v>5459</v>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>+1703</t>
+          <t>+1763</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-09 05:00:12
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -53,6 +53,7 @@
     <sheet name="2026-09-06" sheetId="44" state="visible" r:id="rId44"/>
     <sheet name="2026-09-07" sheetId="45" state="visible" r:id="rId45"/>
     <sheet name="2026-09-08" sheetId="46" state="visible" r:id="rId46"/>
+    <sheet name="2026-09-09" sheetId="47" state="visible" r:id="rId47"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -36886,6 +36887,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet47.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105) | S64</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-09 13:00:11</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>20039</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>$ p i r i t</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>379</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>+20</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Harimukun</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>NAOR</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>6372</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>+540</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>130</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>9258</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>+2032</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>£_Darkz_£</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>AstreaEX</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>820</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Tobi</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>KOSAKI</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>PRINCE G™</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>2091</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>+1588</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>ProfessorX ?</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>696</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>+70</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>ASHBORN™</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Devia Ayu</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>3126</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>1023</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Ryujin Senju™</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>28259</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+2207</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>ZenithEX</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>15729</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>+1320</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>MERU™</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>25924</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>+2300</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Signature</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Sesshomaru</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>+10</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>King Fortuners</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>1203</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Raiden</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>420</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Hail AangEX</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>15162</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Kokyotosu</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>3364</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>+1104</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Arya</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Stüssy</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>5622</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>29815</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>+2980</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>672</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>+302</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>25210</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+2962</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>7643</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>+2184</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>184</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-09 05:30:28
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -36917,11 +36917,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-09 13:00:11</t>
+          <t>Timestamp: 2026-09-09 13:30:27</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>20039</v>
+        <v>541</v>
       </c>
     </row>
     <row r="3">
@@ -37203,11 +37203,11 @@
         </is>
       </c>
       <c r="B21" s="3" t="n">
-        <v>2091</v>
+        <v>2151</v>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>+1588</t>
+          <t>+1648</t>
         </is>
       </c>
     </row>
@@ -37233,11 +37233,11 @@
         </is>
       </c>
       <c r="B23" s="3" t="n">
-        <v>696</v>
+        <v>996</v>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>+70</t>
+          <t>+370</t>
         </is>
       </c>
     </row>
@@ -37353,11 +37353,11 @@
         </is>
       </c>
       <c r="B31" s="3" t="n">
-        <v>28259</v>
+        <v>28283</v>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>+2207</t>
+          <t>+2231</t>
         </is>
       </c>
     </row>
@@ -37368,11 +37368,11 @@
         </is>
       </c>
       <c r="B32" s="3" t="n">
-        <v>15729</v>
+        <v>15789</v>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>+1320</t>
+          <t>+1380</t>
         </is>
       </c>
     </row>
@@ -37668,11 +37668,11 @@
         </is>
       </c>
       <c r="B52" s="3" t="n">
-        <v>29815</v>
+        <v>29875</v>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>+2980</t>
+          <t>+3040</t>
         </is>
       </c>
     </row>
@@ -37713,11 +37713,11 @@
         </is>
       </c>
       <c r="B55" s="3" t="n">
-        <v>25210</v>
+        <v>25270</v>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>+2962</t>
+          <t>+3022</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-10 05:00:09
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -54,6 +54,7 @@
     <sheet name="2026-09-07" sheetId="45" state="visible" r:id="rId45"/>
     <sheet name="2026-09-08" sheetId="46" state="visible" r:id="rId46"/>
     <sheet name="2026-09-09" sheetId="47" state="visible" r:id="rId47"/>
+    <sheet name="2026-09-10" sheetId="48" state="visible" r:id="rId48"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -37775,6 +37776,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105) | S64</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-10 13:00:07</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>20438</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>$ p i r i t</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>379</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Harimukun</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>NAOR</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>6672</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>140</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>+10</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>10338</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>+1080</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>£_Darkz_£</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>AstreaEX</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>820</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Tobi</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>KOSAKI</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>PRINCE G™</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>3549</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>+1398</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>ProfessorX ?</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>1188</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>+192</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>C.L.A.Z</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Devia Ayu</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>4197</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>+1071</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>1023</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Ryujin Senju™</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>30227</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+1944</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>ZenithEX</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>18015</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>+2226</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>MERU™</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>27838</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>+1914</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Signature</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Sesshomaru</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>King Fortuners</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>2271</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>+1068</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Raiden</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>420</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Breaker</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>15162</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Kokyotosu</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>4528</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>+1164</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Arya</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Stüssy</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>5922</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>32695</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>+2820</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>672</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>27040</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+1770</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>9983</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>+2340</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>484</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-10 05:30:30
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -37806,11 +37806,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-10 13:00:07</t>
+          <t>Timestamp: 2026-09-10 13:30:25</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>20438</v>
+        <v>240</v>
       </c>
     </row>
     <row r="3">
@@ -38242,11 +38242,11 @@
         </is>
       </c>
       <c r="B31" s="3" t="n">
-        <v>30227</v>
+        <v>30287</v>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>+1944</t>
+          <t>+2004</t>
         </is>
       </c>
     </row>
@@ -38257,11 +38257,11 @@
         </is>
       </c>
       <c r="B32" s="3" t="n">
-        <v>18015</v>
+        <v>18075</v>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>+2226</t>
+          <t>+2286</t>
         </is>
       </c>
     </row>
@@ -38557,11 +38557,11 @@
         </is>
       </c>
       <c r="B52" s="3" t="n">
-        <v>32695</v>
+        <v>32755</v>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>+2820</t>
+          <t>+2880</t>
         </is>
       </c>
     </row>
@@ -38602,11 +38602,11 @@
         </is>
       </c>
       <c r="B55" s="3" t="n">
-        <v>27040</v>
+        <v>27100</v>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>+1770</t>
+          <t>+1830</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-11 05:00:12
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -55,6 +55,7 @@
     <sheet name="2026-09-08" sheetId="46" state="visible" r:id="rId46"/>
     <sheet name="2026-09-09" sheetId="47" state="visible" r:id="rId47"/>
     <sheet name="2026-09-10" sheetId="48" state="visible" r:id="rId48"/>
+    <sheet name="2026-09-11" sheetId="49" state="visible" r:id="rId49"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -38664,6 +38665,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105) | S64</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-11 13:00:11</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>21389</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>$ p i r i t</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>379</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Harimukun</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>NAOR</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>6672</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>150</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>+10</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>1782</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>+1782</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>12008</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>+1670</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>£_Darkz_£</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>AstreaEX</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>1828</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>+1800</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>820</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>1644</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>+1644</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Tobi</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>KOSAKI</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>PRINCE G™</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>5694</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>+2145</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>ProfessorX ?</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>1188</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>C.L.A.Z</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Devia Ayu</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>5397</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>+1200</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>1023</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Ryujin Senju™</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>32219</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+1932</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>ZenithEX</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>19386</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>+1311</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>MERU™</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>29920</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>+2082</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Signature</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Sesshomaru</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>King Fortuners</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>2631</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>+360</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Raiden</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>420</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Breaker</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>15162</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Kokyotosu</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>4528</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Arya</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Stüssy</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>6222</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>35575</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>+2820</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>672</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>28893</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+1793</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>10283</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>484</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-11 05:30:28
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -38695,11 +38695,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-11 13:00:11</t>
+          <t>Timestamp: 2026-09-11 13:30:26</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>21389</v>
+        <v>356</v>
       </c>
     </row>
     <row r="3">
@@ -38801,11 +38801,11 @@
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>1782</v>
+        <v>1842</v>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>+1782</t>
+          <t>+1842</t>
         </is>
       </c>
     </row>
@@ -38816,11 +38816,11 @@
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>12008</v>
+        <v>12068</v>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>+1670</t>
+          <t>+1730</t>
         </is>
       </c>
     </row>
@@ -38846,11 +38846,11 @@
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>1828</v>
+        <v>1888</v>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>+1800</t>
+          <t>+1860</t>
         </is>
       </c>
     </row>
@@ -38891,11 +38891,11 @@
         </is>
       </c>
       <c r="B15" s="3" t="n">
-        <v>1644</v>
+        <v>1650</v>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>+1644</t>
+          <t>+1650</t>
         </is>
       </c>
     </row>
@@ -39026,11 +39026,11 @@
         </is>
       </c>
       <c r="B24" s="3" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+50</t>
         </is>
       </c>
     </row>
@@ -39446,11 +39446,11 @@
         </is>
       </c>
       <c r="B52" s="3" t="n">
-        <v>35575</v>
+        <v>35635</v>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>+2820</t>
+          <t>+2880</t>
         </is>
       </c>
     </row>
@@ -39491,11 +39491,11 @@
         </is>
       </c>
       <c r="B55" s="3" t="n">
-        <v>28893</v>
+        <v>28953</v>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>+1793</t>
+          <t>+1853</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-12 05:00:10
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -56,6 +56,7 @@
     <sheet name="2026-09-09" sheetId="47" state="visible" r:id="rId47"/>
     <sheet name="2026-09-10" sheetId="48" state="visible" r:id="rId48"/>
     <sheet name="2026-09-11" sheetId="49" state="visible" r:id="rId49"/>
+    <sheet name="2026-09-12" sheetId="50" state="visible" r:id="rId50"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -40441,6 +40442,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet50.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105) | S64</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-12 13:00:09</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>19037</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>$ p i r i t</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>379</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Harimukun</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>NAOR</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>6672</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>150</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>2382</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>+540</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>13808</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>+1740</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>£_Darkz_£</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>AstreaEX</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>4489</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>+2601</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>820</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>4194</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>+2544</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Tobi</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>KOSAKI</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>PRINCE G™</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>5834</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>+140</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>MeiMei</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>1228</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>C.L.A.Z</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Devia Ayu</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>6474</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>+1077</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>1023</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Ryujin Senju™</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>33710</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+1491</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>ZenithEX</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>19890</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>+504</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>MERU™</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>31261</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>+1341</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Signature</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Sesshomaru</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>King Fortuners</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>3633</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>+1002</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Raiden</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>420</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Breaker</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>15162</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Kokyotosu</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>4528</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Arya</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Stüssy</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>6322</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>37965</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>+2330</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>672</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>31584</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+2631</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>10283</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>1084</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-12 05:30:24
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -40472,11 +40472,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-12 13:00:09</t>
+          <t>Timestamp: 2026-09-12 13:30:23</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>19037</v>
+        <v>221</v>
       </c>
     </row>
     <row r="3">
@@ -41223,11 +41223,11 @@
         </is>
       </c>
       <c r="B52" s="3" t="n">
-        <v>37965</v>
+        <v>38085</v>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>+2330</t>
+          <t>+2450</t>
         </is>
       </c>
     </row>
@@ -41268,11 +41268,11 @@
         </is>
       </c>
       <c r="B55" s="3" t="n">
-        <v>31584</v>
+        <v>31685</v>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>+2631</t>
+          <t>+2732</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-13 05:00:12
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -57,6 +57,7 @@
     <sheet name="2026-09-10" sheetId="48" state="visible" r:id="rId48"/>
     <sheet name="2026-09-11" sheetId="49" state="visible" r:id="rId49"/>
     <sheet name="2026-09-12" sheetId="50" state="visible" r:id="rId50"/>
+    <sheet name="2026-09-13" sheetId="51" state="visible" r:id="rId51"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -41330,6 +41331,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet51.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105) | S64</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-13 13:00:11</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>25556</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>$ p i r i t</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>379</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Harimukun</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>NAOR</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>6672</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>150</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>2975</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>+593</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>17504</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>+3696</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>£_Darkz_£</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>820</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>ZÎ£ WHITÎ£BÎ£ARD</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>AangEX2</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>5520</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Khakashi Hatake</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>KOSAKI</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>PRINCE G™</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>8409</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>+2575</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>el MeiMei</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>2072</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>C.L.A.Z</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Devia Ayu</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>6474</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>1023</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Ryujin Senju™</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>34550</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>+840</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>ZenithEX</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>21360</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>+1470</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>MERU™</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>32101</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>+840</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>SNC | $ignature</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Sesshomaru</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>King Fortuners</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>5074</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>+1441</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Raiden</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>420</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Breaker</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>16002</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>+840</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Kokyotosu</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>4528</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Arya</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Stüssy</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>7162</v>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>+840</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n">
+        <v>44877</v>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>+6792</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n">
+        <v>672</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="n">
+        <v>34923</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>+3238</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n">
+        <v>10283</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="n">
+        <v>1084</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-13 05:30:35
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -41361,11 +41361,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-13 13:00:11</t>
+          <t>Timestamp: 2026-09-13 13:30:34</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>25556</v>
+        <v>168</v>
       </c>
     </row>
     <row r="3">
@@ -42112,11 +42112,11 @@
         </is>
       </c>
       <c r="B52" s="3" t="n">
-        <v>44877</v>
+        <v>45045</v>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>+6792</t>
+          <t>+6960</t>
         </is>
       </c>
     </row>

</xml_diff>